<commit_message>
Sync input template workbooks to Chinese column labels
Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inputs/template_cn.xlsx
+++ b/inputs/template_cn.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-38520" yWindow="5100" windowWidth="38640" windowHeight="21240" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="概览" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="经济工具" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="工具总览" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="规制工具" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="政府投资与消费" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="信息工具" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="自愿措施" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="封面" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="分类框架" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="类别与组别" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="属性定义" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="已终止" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概览" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="经济工具" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工具总览" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规制工具" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="政府投资与消费" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="信息工具" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="自愿措施" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="封面" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分类框架" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="类别与组别" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="属性定义" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="已终止" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -799,7 +799,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="34">
+  <borders count="39">
     <border>
       <left/>
       <right/>
@@ -1132,16 +1132,16 @@
     </border>
     <border>
       <left style="thin">
-        <color auto="Values must be of type &lt;class 'bool'&gt;"/>
+        <color auto="1"/>
       </left>
       <right style="thin">
-        <color auto="Values must be of type &lt;class 'bool'&gt;"/>
+        <color auto="1"/>
       </right>
       <top style="thin">
-        <color auto="Values must be of type &lt;class 'bool'&gt;"/>
+        <color auto="1"/>
       </top>
       <bottom style="thin">
-        <color auto="Values must be of type &lt;class 'bool'&gt;"/>
+        <color auto="1"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1149,46 +1149,95 @@
       <left/>
       <right/>
       <top style="thin">
-        <color auto="Values must be of type &lt;class 'bool'&gt;"/>
+        <color auto="1"/>
       </top>
       <bottom style="thin">
-        <color auto="Values must be of type &lt;class 'bool'&gt;"/>
+        <color auto="1"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left/>
       <right style="thin">
-        <color auto="Values must be of type &lt;class 'bool'&gt;"/>
+        <color auto="1"/>
       </right>
       <top style="thin">
-        <color auto="Values must be of type &lt;class 'bool'&gt;"/>
+        <color auto="1"/>
       </top>
       <bottom style="thin">
-        <color auto="Values must be of type &lt;class 'bool'&gt;"/>
+        <color auto="1"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color auto="Values must be of type &lt;class 'bool'&gt;"/>
+        <color auto="1"/>
       </left>
       <right style="thin">
-        <color auto="Values must be of type &lt;class 'bool'&gt;"/>
+        <color auto="1"/>
       </right>
       <top/>
       <bottom style="thin">
-        <color auto="Values must be of type &lt;class 'bool'&gt;"/>
+        <color auto="1"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color auto="Values must be of type &lt;class 'bool'&gt;"/>
+        <color auto="1"/>
       </left>
       <right style="thin">
-        <color auto="Values must be of type &lt;class 'bool'&gt;"/>
+        <color auto="1"/>
       </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
       <top/>
       <bottom/>
       <diagonal/>
@@ -3224,7 +3273,7 @@
       </c>
       <c r="N39" s="100" t="inlineStr">
         <is>
-          <t>总计</t>
+          <t>路径数量总计</t>
         </is>
       </c>
     </row>
@@ -15883,8 +15932,8 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A3:B3"/>
     <mergeCell ref="A8:A9"/>
-    <mergeCell ref="A3:B3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Normalize Agent to enumeration, rework Objective vocabulary, translate EN ended row
- Consolidate Agent (受规制主体) to the 4-value enumeration (家庭/企业/政府/非政府组织; Households/Firms/Governments/Non-governmental organisations) across all CN/EN rows with per-row CN/EN alignment
- Rework Objective to a 17-term vocabulary: merge 节能 into 能源效率, 资源节约 into 循环经济, 可再生能源发展 into new 非化石能源, biodiversity/desertification terms into 生态保护; drop employment and poverty reduction, public health, food safety and capacity building; add 非化石能源, 绿色金融 and 电气化 with row backfill and evidence entries
- Update schema, templates, attribute definitions and field dictionary to the new Objective vocabulary
- Translate remaining Chinese fields in the EN ended CSV (EPC VAT incentive)
</commit_message>
<xml_diff>
--- a/inputs/template_cn.xlsx
+++ b/inputs/template_cn.xlsx
@@ -5488,7 +5488,7 @@
       </c>
       <c r="E12" s="372" t="inlineStr">
         <is>
-          <t>空气污染；废弃物减量/循环经济；减缓气候变化；适应气候变化；经济增长；能源效率；能源安全；社会保障/减贫；其他；未指明</t>
+          <t>减缓气候变化；非化石能源；能源效率；绿色经济；技术创新；能源安全；污染防治；生态保护；循环经济；适应气候变化；绿色金融；电气化；产业发展；绿色消费；信息披露；公众意识；保护臭氧层</t>
         </is>
       </c>
       <c r="F12" s="383" t="n"/>
@@ -11246,13 +11246,13 @@
           <t>中国气候政策工具数据库（CCPID）</t>
         </is>
       </c>
-      <c r="B1" s="425" t="n"/>
-      <c r="C1" s="425" t="n"/>
-      <c r="D1" s="425" t="n"/>
-      <c r="E1" s="425" t="n"/>
-      <c r="F1" s="425" t="n"/>
-      <c r="G1" s="425" t="n"/>
-      <c r="H1" s="426" t="n"/>
+      <c r="B1" s="103" t="n"/>
+      <c r="C1" s="103" t="n"/>
+      <c r="D1" s="103" t="n"/>
+      <c r="E1" s="103" t="n"/>
+      <c r="F1" s="103" t="n"/>
+      <c r="G1" s="103" t="n"/>
+      <c r="H1" s="104" t="n"/>
       <c r="I1" s="427" t="n"/>
       <c r="J1" s="427" t="n"/>
       <c r="K1" s="428" t="n"/>

</xml_diff>

<commit_message>
Drop Country column, remove superseded beer standard row, fix ISIC and mitigation relevance, capture EN Cover edits
- Remove Country field from schema, templates, scripts, docs, and all CSVs
- Delete superseded GB 32047-2015 row; keep GB 32047-2025 row with predecessor dates and old version mentioned in descriptions
- Fix ISIC economic sector values in voluntary approaches
- Recode carbon-efficiency top-runner mitigation relevance to Direct
- Capture EN Cover rows 3/7 formatting edits into template_en.xlsx
- Regenerate workbooks and webpages

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inputs/template_cn.xlsx
+++ b/inputs/template_cn.xlsx
@@ -5038,7 +5038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T95"/>
+  <dimension ref="A1:T94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34.46875" customWidth="1" min="1" max="1"/>
@@ -5549,12 +5549,12 @@
       <c r="A14" s="293" t="n"/>
       <c r="B14" s="371" t="inlineStr">
         <is>
-          <t>国家</t>
+          <t>管辖层级</t>
         </is>
       </c>
       <c r="C14" s="371" t="inlineStr">
         <is>
-          <t>该政策工具适用的国家</t>
+          <t>该工具适用的管辖层级</t>
         </is>
       </c>
       <c r="D14" s="372" t="inlineStr">
@@ -5564,7 +5564,7 @@
       </c>
       <c r="E14" s="372" t="inlineStr">
         <is>
-          <t>IFCMA成员国家清单</t>
+          <t>国家级；次国家级；超国家级；经济特区</t>
         </is>
       </c>
       <c r="F14" s="383" t="n"/>
@@ -5587,22 +5587,22 @@
       <c r="A15" s="293" t="n"/>
       <c r="B15" s="371" t="inlineStr">
         <is>
-          <t>管辖层级</t>
+          <t>管辖地名称</t>
         </is>
       </c>
       <c r="C15" s="371" t="inlineStr">
         <is>
-          <t>该工具适用的管辖层级</t>
+          <t>若工具在超国家/国际层级或次国家级适用，填写管辖地名称（以英文填写）</t>
         </is>
       </c>
       <c r="D15" s="372" t="inlineStr">
         <is>
-          <t>分类（单选）</t>
+          <t>自由文本</t>
         </is>
       </c>
       <c r="E15" s="372" t="inlineStr">
         <is>
-          <t>国家级；次国家级；超国家级；经济特区</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="F15" s="383" t="n"/>
@@ -5625,22 +5625,22 @@
       <c r="A16" s="293" t="n"/>
       <c r="B16" s="371" t="inlineStr">
         <is>
-          <t>管辖地名称</t>
+          <t>状态</t>
         </is>
       </c>
       <c r="C16" s="371" t="inlineStr">
         <is>
-          <t>若工具在超国家/国际层级或次国家级适用，填写管辖地名称（以英文填写）</t>
+          <t>界定该工具是现行有效还是已失效，以及是否正在生效</t>
         </is>
       </c>
       <c r="D16" s="372" t="inlineStr">
         <is>
-          <t>自由文本</t>
+          <t>分类（单选）</t>
         </is>
       </c>
       <c r="E16" s="372" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>生效；计划实施；已终止；不存在</t>
         </is>
       </c>
       <c r="F16" s="383" t="n"/>
@@ -5663,22 +5663,22 @@
       <c r="A17" s="293" t="n"/>
       <c r="B17" s="371" t="inlineStr">
         <is>
-          <t>状态</t>
+          <t>通过日期</t>
         </is>
       </c>
       <c r="C17" s="371" t="inlineStr">
         <is>
-          <t>界定该工具是现行有效还是已失效，以及是否正在生效</t>
+          <t>该工具获批的日期</t>
         </is>
       </c>
       <c r="D17" s="372" t="inlineStr">
         <is>
-          <t>分类（单选）</t>
+          <t>日月年格式</t>
         </is>
       </c>
       <c r="E17" s="372" t="inlineStr">
         <is>
-          <t>生效；计划实施；已终止；不存在</t>
+          <t>固定格式 [mm/yyyy] 或 [yyyy]</t>
         </is>
       </c>
       <c r="F17" s="383" t="n"/>
@@ -5701,12 +5701,12 @@
       <c r="A18" s="293" t="n"/>
       <c r="B18" s="371" t="inlineStr">
         <is>
-          <t>通过日期</t>
+          <t>生效日期</t>
         </is>
       </c>
       <c r="C18" s="371" t="inlineStr">
         <is>
-          <t>该工具获批的日期</t>
+          <t>该工具生效或即将生效、具有法律约束力的日期</t>
         </is>
       </c>
       <c r="D18" s="372" t="inlineStr">
@@ -5739,12 +5739,12 @@
       <c r="A19" s="293" t="n"/>
       <c r="B19" s="371" t="inlineStr">
         <is>
-          <t>生效日期</t>
+          <t>终止日期</t>
         </is>
       </c>
       <c r="C19" s="371" t="inlineStr">
         <is>
-          <t>该工具生效或即将生效、具有法律约束力的日期</t>
+          <t>法律授权的最终要求生效的日期（如相关）</t>
         </is>
       </c>
       <c r="D19" s="372" t="inlineStr">
@@ -5777,12 +5777,12 @@
       <c r="A20" s="293" t="n"/>
       <c r="B20" s="371" t="inlineStr">
         <is>
-          <t>终止日期</t>
+          <t>最近修订</t>
         </is>
       </c>
       <c r="C20" s="371" t="inlineStr">
         <is>
-          <t>法律授权的最终要求生效的日期（如相关）</t>
+          <t>该政策工具最近一次更新/修订的日期</t>
         </is>
       </c>
       <c r="D20" s="372" t="inlineStr">
@@ -5815,24 +5815,20 @@
       <c r="A21" s="293" t="n"/>
       <c r="B21" s="371" t="inlineStr">
         <is>
-          <t>最近修订</t>
+          <t>最近修订（详情）</t>
         </is>
       </c>
       <c r="C21" s="371" t="inlineStr">
         <is>
-          <t>该政策工具最近一次更新/修订的日期</t>
+          <t>说明最近一次修订的性质（如适用）、修改内容[扩大范围、调整强度、新增专项资金安排等]以及/或此前相关修订</t>
         </is>
       </c>
       <c r="D21" s="372" t="inlineStr">
         <is>
-          <t>日月年格式</t>
-        </is>
-      </c>
-      <c r="E21" s="372" t="inlineStr">
-        <is>
-          <t>固定格式 [mm/yyyy] 或 [yyyy]</t>
-        </is>
-      </c>
+          <t>自由文本</t>
+        </is>
+      </c>
+      <c r="E21" s="372" t="n"/>
       <c r="F21" s="383" t="n"/>
       <c r="G21" s="412" t="n"/>
       <c r="H21" s="412" t="n"/>
@@ -5850,15 +5846,15 @@
       <c r="T21" s="412" t="n"/>
     </row>
     <row r="22" ht="15" customHeight="1">
-      <c r="A22" s="293" t="n"/>
+      <c r="A22" s="282" t="n"/>
       <c r="B22" s="371" t="inlineStr">
         <is>
-          <t>最近修订（详情）</t>
+          <t>管理机构</t>
         </is>
       </c>
       <c r="C22" s="371" t="inlineStr">
         <is>
-          <t>说明最近一次修订的性质（如适用）、修改内容[扩大范围、调整强度、新增专项资金安排等]以及/或此前相关修订</t>
+          <t>实施和管理该工具的机构。包括设定费率及/或界定政策基础</t>
         </is>
       </c>
       <c r="D22" s="372" t="inlineStr">
@@ -5866,7 +5862,11 @@
           <t>自由文本</t>
         </is>
       </c>
-      <c r="E22" s="372" t="n"/>
+      <c r="E22" s="372" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="F22" s="383" t="n"/>
       <c r="G22" s="412" t="n"/>
       <c r="H22" s="412" t="n"/>
@@ -5884,25 +5884,29 @@
       <c r="T22" s="412" t="n"/>
     </row>
     <row r="23" ht="15" customHeight="1">
-      <c r="A23" s="282" t="n"/>
+      <c r="A23" s="375" t="inlineStr">
+        <is>
+          <t>政策规制基础与强度</t>
+        </is>
+      </c>
       <c r="B23" s="371" t="inlineStr">
         <is>
-          <t>管理机构</t>
+          <t>受规制资产</t>
         </is>
       </c>
       <c r="C23" s="371" t="inlineStr">
         <is>
-          <t>实施和管理该工具的机构。包括设定费率及/或界定政策基础</t>
+          <t>受规制的对象；可以是构筑物（如锅炉和汽轮机）、燃料（如煤炭或天然气）、排放物，也可以是产品、投入品等更一般的对象，以及无形资产</t>
         </is>
       </c>
       <c r="D23" s="372" t="inlineStr">
         <is>
-          <t>自由文本</t>
+          <t>分类（多选），可补充详情</t>
         </is>
       </c>
       <c r="E23" s="372" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>非穷尽清单</t>
         </is>
       </c>
       <c r="F23" s="383" t="n"/>
@@ -5922,29 +5926,25 @@
       <c r="T23" s="412" t="n"/>
     </row>
     <row r="24" ht="15" customHeight="1">
-      <c r="A24" s="375" t="inlineStr">
-        <is>
-          <t>政策规制基础与强度</t>
-        </is>
-      </c>
+      <c r="A24" s="293" t="n"/>
       <c r="B24" s="371" t="inlineStr">
         <is>
-          <t>受规制资产</t>
+          <t>受规制资产（状态）</t>
         </is>
       </c>
       <c r="C24" s="371" t="inlineStr">
         <is>
-          <t>受规制的对象；可以是构筑物（如锅炉和汽轮机）、燃料（如煤炭或天然气）、排放物，也可以是产品、投入品等更一般的对象，以及无形资产</t>
+          <t>资产状态，即资产是新建/新售的、已存在的（既有建筑存量或车辆存量），还是二手售出的</t>
         </is>
       </c>
       <c r="D24" s="372" t="inlineStr">
         <is>
-          <t>分类（多选），可补充详情</t>
+          <t>分类</t>
         </is>
       </c>
       <c r="E24" s="372" t="inlineStr">
         <is>
-          <t>非穷尽清单</t>
+          <t>新建；既有</t>
         </is>
       </c>
       <c r="F24" s="383" t="n"/>
@@ -5967,12 +5967,12 @@
       <c r="A25" s="293" t="n"/>
       <c r="B25" s="371" t="inlineStr">
         <is>
-          <t>受规制资产（状态）</t>
+          <t>受规制资产（详情）</t>
         </is>
       </c>
       <c r="C25" s="371" t="inlineStr">
         <is>
-          <t>资产状态，即资产是新建/新售的、已存在的（既有建筑存量或车辆存量），还是二手售出的</t>
+          <t>资产类型，视资产种类可有多种形式，可包括发动机类型或其他技术规格</t>
         </is>
       </c>
       <c r="D25" s="372" t="inlineStr">
@@ -5982,7 +5982,7 @@
       </c>
       <c r="E25" s="372" t="inlineStr">
         <is>
-          <t>新建；既有</t>
+          <t>非穷尽清单</t>
         </is>
       </c>
       <c r="F25" s="383" t="n"/>
@@ -6005,22 +6005,22 @@
       <c r="A26" s="293" t="n"/>
       <c r="B26" s="371" t="inlineStr">
         <is>
-          <t>受规制资产（详情）</t>
+          <t>受规制资产（其他）</t>
         </is>
       </c>
       <c r="C26" s="371" t="inlineStr">
         <is>
-          <t>资产类型，视资产种类可有多种形式，可包括发动机类型或其他技术规格</t>
+          <t>界定受规制资产所需的其他详情</t>
         </is>
       </c>
       <c r="D26" s="372" t="inlineStr">
         <is>
-          <t>分类</t>
+          <t>自由文本</t>
         </is>
       </c>
       <c r="E26" s="372" t="inlineStr">
         <is>
-          <t>非穷尽清单</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="F26" s="383" t="n"/>
@@ -6043,22 +6043,22 @@
       <c r="A27" s="293" t="n"/>
       <c r="B27" s="371" t="inlineStr">
         <is>
-          <t>受规制资产（其他）</t>
+          <t>受规制资产（阈值范围）</t>
         </is>
       </c>
       <c r="C27" s="371" t="inlineStr">
         <is>
-          <t>界定受规制资产所需的其他详情</t>
+          <t>指界定该工具所规制的政策基础范围或类别的具体详情。括号划定该工具规制条款适用的边界，例如收入区间、资产类别（如按规模划分）。</t>
         </is>
       </c>
       <c r="D27" s="372" t="inlineStr">
         <is>
-          <t>自由文本</t>
+          <t>开放结构</t>
         </is>
       </c>
       <c r="E27" s="372" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>[XXXX ; YYYY] + 单位</t>
         </is>
       </c>
       <c r="F27" s="383" t="n"/>
@@ -6081,22 +6081,22 @@
       <c r="A28" s="293" t="n"/>
       <c r="B28" s="371" t="inlineStr">
         <is>
-          <t>受规制资产（阈值范围）</t>
+          <t>受规制主体</t>
         </is>
       </c>
       <c r="C28" s="371" t="inlineStr">
         <is>
-          <t>指界定该工具所规制的政策基础范围或类别的具体详情。括号划定该工具规制条款适用的边界，例如收入区间、资产类别（如按规模划分）。</t>
+          <t>依法须遵守该政策工具，或获得既定利益或信息的主体</t>
         </is>
       </c>
       <c r="D28" s="372" t="inlineStr">
         <is>
-          <t>开放结构</t>
+          <t>分类（多选），可补充详情</t>
         </is>
       </c>
       <c r="E28" s="372" t="inlineStr">
         <is>
-          <t>[XXXX ; YYYY] + 单位</t>
+          <t>家庭；企业；政府；非政府组织</t>
         </is>
       </c>
       <c r="F28" s="383" t="n"/>
@@ -6119,22 +6119,22 @@
       <c r="A29" s="293" t="n"/>
       <c r="B29" s="371" t="inlineStr">
         <is>
-          <t>受规制主体</t>
+          <t>受规制主体（详情）</t>
         </is>
       </c>
       <c r="C29" s="371" t="inlineStr">
         <is>
-          <t>依法须遵守该政策工具，或获得既定利益或信息的主体</t>
+          <t>界定受规制主体所需的相关详情（例如：车龄超过10年的车辆、收入超过一定门槛的家庭/企业等）</t>
         </is>
       </c>
       <c r="D29" s="372" t="inlineStr">
         <is>
-          <t>分类（多选），可补充详情</t>
+          <t>自由文本</t>
         </is>
       </c>
       <c r="E29" s="372" t="inlineStr">
         <is>
-          <t>家庭；企业；政府；非政府组织</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="F29" s="383" t="n"/>
@@ -6157,22 +6157,22 @@
       <c r="A30" s="293" t="n"/>
       <c r="B30" s="371" t="inlineStr">
         <is>
-          <t>受规制主体（详情）</t>
+          <t>受规制活动</t>
         </is>
       </c>
       <c r="C30" s="371" t="inlineStr">
         <is>
-          <t>界定受规制主体所需的相关详情（例如：车龄超过10年的车辆、收入超过一定门槛的家庭/企业等）</t>
+          <t>该政策工具干预的作用点</t>
         </is>
       </c>
       <c r="D30" s="372" t="inlineStr">
         <is>
-          <t>自由文本</t>
+          <t>分类（多选），可补充详情</t>
         </is>
       </c>
       <c r="E30" s="372" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>非穷尽清单</t>
         </is>
       </c>
       <c r="F30" s="383" t="n"/>
@@ -6195,22 +6195,22 @@
       <c r="A31" s="293" t="n"/>
       <c r="B31" s="371" t="inlineStr">
         <is>
-          <t>受规制活动</t>
+          <t>受规制活动（详情）</t>
         </is>
       </c>
       <c r="C31" s="371" t="inlineStr">
         <is>
-          <t>该政策工具干预的作用点</t>
+          <t>界定受规制活动所需的其他详情</t>
         </is>
       </c>
       <c r="D31" s="372" t="inlineStr">
         <is>
-          <t>分类（多选），可补充详情</t>
+          <t>自由文本</t>
         </is>
       </c>
       <c r="E31" s="372" t="inlineStr">
         <is>
-          <t>非穷尽清单</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="F31" s="383" t="n"/>
@@ -6233,12 +6233,12 @@
       <c r="A32" s="293" t="n"/>
       <c r="B32" s="371" t="inlineStr">
         <is>
-          <t>受规制活动（详情）</t>
+          <t>强度（数值）</t>
         </is>
       </c>
       <c r="C32" s="371" t="inlineStr">
         <is>
-          <t>界定受规制活动所需的其他详情</t>
+          <t>法律文件中使用的数值（水平、费率、目标等）</t>
         </is>
       </c>
       <c r="D32" s="372" t="inlineStr">
@@ -6271,12 +6271,12 @@
       <c r="A33" s="293" t="n"/>
       <c r="B33" s="371" t="inlineStr">
         <is>
-          <t>强度（数值）</t>
+          <t>强度（单位）</t>
         </is>
       </c>
       <c r="C33" s="371" t="inlineStr">
         <is>
-          <t>法律文件中使用的数值（水平、费率、目标等）</t>
+          <t>强度数值的单位，例如：欧元、公里、%、等级等</t>
         </is>
       </c>
       <c r="D33" s="372" t="inlineStr">
@@ -6286,7 +6286,7 @@
       </c>
       <c r="E33" s="372" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>[按法规中所述的单位填写]</t>
         </is>
       </c>
       <c r="F33" s="383" t="n"/>
@@ -6309,12 +6309,12 @@
       <c r="A34" s="293" t="n"/>
       <c r="B34" s="371" t="inlineStr">
         <is>
-          <t>强度（单位）</t>
+          <t>强度（详情）</t>
         </is>
       </c>
       <c r="C34" s="371" t="inlineStr">
         <is>
-          <t>强度数值的单位，例如：欧元、公里、%、等级等</t>
+          <t>关于强度的进一步详情（如需要）。例如：若强度按公式计算，可提供公式及平均强度值</t>
         </is>
       </c>
       <c r="D34" s="372" t="inlineStr">
@@ -6324,7 +6324,7 @@
       </c>
       <c r="E34" s="372" t="inlineStr">
         <is>
-          <t>[按法规中所述的单位填写]</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="F34" s="383" t="n"/>
@@ -6347,12 +6347,12 @@
       <c r="A35" s="293" t="n"/>
       <c r="B35" s="371" t="inlineStr">
         <is>
-          <t>强度（详情）</t>
+          <t>要求说明</t>
         </is>
       </c>
       <c r="C35" s="371" t="inlineStr">
         <is>
-          <t>关于强度的进一步详情（如需要）。例如：若强度按公式计算，可提供公式及平均强度值</t>
+          <t>若强度因某项尚未在资产、活动或主体属性中体现的要求而变化，且该要求对理解和描述该政策工具有意义，则在此填写该项要求。</t>
         </is>
       </c>
       <c r="D35" s="372" t="inlineStr">
@@ -6385,12 +6385,12 @@
       <c r="A36" s="293" t="n"/>
       <c r="B36" s="371" t="inlineStr">
         <is>
-          <t>要求说明</t>
+          <t>合规计算方法I</t>
         </is>
       </c>
       <c r="C36" s="371" t="inlineStr">
         <is>
-          <t>若强度因某项尚未在资产、活动或主体属性中体现的要求而变化，且该要求对理解和描述该政策工具有意义，则在此填写该项要求。</t>
+          <t>指明该工具适用于单个受规制资产，还是资产的加总（例如其总产量、总运营量或总销量）。</t>
         </is>
       </c>
       <c r="D36" s="372" t="inlineStr">
@@ -6420,15 +6420,15 @@
       <c r="T36" s="412" t="n"/>
     </row>
     <row r="37" ht="15" customHeight="1">
-      <c r="A37" s="293" t="n"/>
+      <c r="A37" s="282" t="n"/>
       <c r="B37" s="371" t="inlineStr">
         <is>
-          <t>合规计算方法I</t>
+          <t>合规计算方法II</t>
         </is>
       </c>
       <c r="C37" s="371" t="inlineStr">
         <is>
-          <t>指明该工具适用于单个受规制资产，还是资产的加总（例如其总产量、总运营量或总销量）。</t>
+          <t>描述用于评估是否满足该工具要求的方法或规则。</t>
         </is>
       </c>
       <c r="D37" s="372" t="inlineStr">
@@ -6458,15 +6458,19 @@
       <c r="T37" s="412" t="n"/>
     </row>
     <row r="38" ht="15" customHeight="1">
-      <c r="A38" s="282" t="n"/>
+      <c r="A38" s="375" t="inlineStr">
+        <is>
+          <t>立法参考</t>
+        </is>
+      </c>
       <c r="B38" s="371" t="inlineStr">
         <is>
-          <t>合规计算方法II</t>
+          <t>法律文件名称</t>
         </is>
       </c>
       <c r="C38" s="371" t="inlineStr">
         <is>
-          <t>描述用于评估是否满足该工具要求的方法或规则。</t>
+          <t>设立或（修订后）修改该工具的相关法律文件名称及章和/或条款</t>
         </is>
       </c>
       <c r="D38" s="372" t="inlineStr">
@@ -6496,19 +6500,15 @@
       <c r="T38" s="412" t="n"/>
     </row>
     <row r="39" ht="15" customHeight="1">
-      <c r="A39" s="375" t="inlineStr">
-        <is>
-          <t>立法参考</t>
-        </is>
-      </c>
+      <c r="A39" s="293" t="n"/>
       <c r="B39" s="371" t="inlineStr">
         <is>
-          <t>法律文件名称</t>
+          <t>法律文件链接</t>
         </is>
       </c>
       <c r="C39" s="371" t="inlineStr">
         <is>
-          <t>设立或（修订后）修改该工具的相关法律文件名称及章和/或条款</t>
+          <t>设立或（修订后）修改该工具的相关法律文件网页链接</t>
         </is>
       </c>
       <c r="D39" s="372" t="inlineStr">
@@ -6538,15 +6538,15 @@
       <c r="T39" s="412" t="n"/>
     </row>
     <row r="40" ht="15" customHeight="1">
-      <c r="A40" s="293" t="n"/>
+      <c r="A40" s="282" t="n"/>
       <c r="B40" s="371" t="inlineStr">
         <is>
-          <t>法律文件链接</t>
+          <t>其他网页链接</t>
         </is>
       </c>
       <c r="C40" s="371" t="inlineStr">
         <is>
-          <t>设立或（修订后）修改该工具的相关法律文件网页链接</t>
+          <t>其他相关网站的网页链接</t>
         </is>
       </c>
       <c r="D40" s="372" t="inlineStr">
@@ -6576,31 +6576,35 @@
       <c r="T40" s="412" t="n"/>
     </row>
     <row r="41" ht="15" customHeight="1">
-      <c r="A41" s="282" t="n"/>
+      <c r="A41" s="375" t="inlineStr">
+        <is>
+          <t>温室气体排放基础</t>
+        </is>
+      </c>
       <c r="B41" s="371" t="inlineStr">
         <is>
-          <t>其他网页链接</t>
+          <t>温室气体排放覆盖（绝对量）</t>
         </is>
       </c>
       <c r="C41" s="371" t="inlineStr">
         <is>
-          <t>其他相关网站的网页链接</t>
+          <t>该工具排放基数（覆盖的排放量）的绝对值量化</t>
         </is>
       </c>
       <c r="D41" s="372" t="inlineStr">
         <is>
-          <t>自由文本</t>
+          <t>数值</t>
         </is>
       </c>
       <c r="E41" s="372" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F41" s="383" t="n"/>
-      <c r="G41" s="412" t="n"/>
-      <c r="H41" s="412" t="n"/>
-      <c r="I41" s="412" t="n"/>
+          <t>单位：千吨CO2当量</t>
+        </is>
+      </c>
+      <c r="F41" s="413" t="n"/>
+      <c r="G41" s="414" t="n"/>
+      <c r="H41" s="414" t="n"/>
+      <c r="I41" s="415" t="n"/>
       <c r="J41" s="412" t="n"/>
       <c r="K41" s="412" t="n"/>
       <c r="L41" s="412" t="n"/>
@@ -6614,19 +6618,15 @@
       <c r="T41" s="412" t="n"/>
     </row>
     <row r="42" ht="15" customHeight="1">
-      <c r="A42" s="375" t="inlineStr">
-        <is>
-          <t>温室气体排放基础</t>
-        </is>
-      </c>
+      <c r="A42" s="282" t="n"/>
       <c r="B42" s="371" t="inlineStr">
         <is>
-          <t>温室气体排放覆盖（绝对量）</t>
+          <t>温室气体排放覆盖（占国内排放百分比）</t>
         </is>
       </c>
       <c r="C42" s="371" t="inlineStr">
         <is>
-          <t>该工具排放基数（覆盖的排放量）的绝对值量化</t>
+          <t>该工具排放基数相对于国内总排放量的量化</t>
         </is>
       </c>
       <c r="D42" s="372" t="inlineStr">
@@ -6636,7 +6636,7 @@
       </c>
       <c r="E42" s="372" t="inlineStr">
         <is>
-          <t>单位：千吨CO2当量</t>
+          <t>占国内排放量的百分比</t>
         </is>
       </c>
       <c r="F42" s="413" t="n"/>
@@ -6656,31 +6656,35 @@
       <c r="T42" s="412" t="n"/>
     </row>
     <row r="43" ht="15" customHeight="1">
-      <c r="A43" s="282" t="n"/>
+      <c r="A43" s="375" t="inlineStr">
+        <is>
+          <t>分类与指标</t>
+        </is>
+      </c>
       <c r="B43" s="371" t="inlineStr">
         <is>
-          <t>温室气体排放覆盖（占国内排放百分比）</t>
+          <t>经济行业</t>
         </is>
       </c>
       <c r="C43" s="371" t="inlineStr">
         <is>
-          <t>该工具排放基数相对于国内总排放量的量化</t>
+          <t>基于受规制主体的分类。若受规制主体为企业，则按《所有经济活动的国际标准行业分类》（ISIC）划分行业</t>
         </is>
       </c>
       <c r="D43" s="372" t="inlineStr">
         <is>
-          <t>数值</t>
+          <t>分类</t>
         </is>
       </c>
       <c r="E43" s="372" t="inlineStr">
         <is>
-          <t>占国内排放量的百分比</t>
-        </is>
-      </c>
-      <c r="F43" s="413" t="n"/>
-      <c r="G43" s="414" t="n"/>
-      <c r="H43" s="414" t="n"/>
-      <c r="I43" s="415" t="n"/>
+          <t>ISIC两位数分类</t>
+        </is>
+      </c>
+      <c r="F43" s="383" t="n"/>
+      <c r="G43" s="412" t="n"/>
+      <c r="H43" s="412" t="n"/>
+      <c r="I43" s="412" t="n"/>
       <c r="J43" s="412" t="n"/>
       <c r="K43" s="412" t="n"/>
       <c r="L43" s="412" t="n"/>
@@ -6694,19 +6698,15 @@
       <c r="T43" s="412" t="n"/>
     </row>
     <row r="44" ht="15" customHeight="1">
-      <c r="A44" s="375" t="inlineStr">
-        <is>
-          <t>分类与指标</t>
-        </is>
-      </c>
+      <c r="A44" s="293" t="n"/>
       <c r="B44" s="371" t="inlineStr">
         <is>
-          <t>经济行业</t>
+          <t>受影响的温室气体</t>
         </is>
       </c>
       <c r="C44" s="371" t="inlineStr">
         <is>
-          <t>基于受规制主体的分类。若受规制主体为企业，则按《所有经济活动的国际标准行业分类》（ISIC）划分行业</t>
+          <t>受规制的温室气体（若直接规制）；否则填写可能受该工具影响的温室气体。</t>
         </is>
       </c>
       <c r="D44" s="372" t="inlineStr">
@@ -6716,7 +6716,7 @@
       </c>
       <c r="E44" s="372" t="inlineStr">
         <is>
-          <t>ISIC两位数分类</t>
+          <t>CO2; CH4; N2O; SF6; HFCs; PFCs; NF3</t>
         </is>
       </c>
       <c r="F44" s="383" t="n"/>
@@ -6739,12 +6739,12 @@
       <c r="A45" s="293" t="n"/>
       <c r="B45" s="371" t="inlineStr">
         <is>
-          <t>受影响的温室气体</t>
+          <t>减缓效果</t>
         </is>
       </c>
       <c r="C45" s="371" t="inlineStr">
         <is>
-          <t>受规制的温室气体（若直接规制）；否则填写可能受该工具影响的温室气体。</t>
+          <t>描述该工具对温室气体排放/碳汇的影响可能为正、为负还是未知</t>
         </is>
       </c>
       <c r="D45" s="372" t="inlineStr">
@@ -6754,7 +6754,7 @@
       </c>
       <c r="E45" s="372" t="inlineStr">
         <is>
-          <t>CO2; CH4; N2O; SF6; HFCs; PFCs; NF3</t>
+          <t>正向；负向；中性；未知</t>
         </is>
       </c>
       <c r="F45" s="383" t="n"/>
@@ -6774,15 +6774,15 @@
       <c r="T45" s="412" t="n"/>
     </row>
     <row r="46" ht="15" customHeight="1">
-      <c r="A46" s="293" t="n"/>
+      <c r="A46" s="282" t="n"/>
       <c r="B46" s="371" t="inlineStr">
         <is>
-          <t>减缓效果</t>
+          <t>减缓协同效益</t>
         </is>
       </c>
       <c r="C46" s="371" t="inlineStr">
         <is>
-          <t>描述该工具对温室气体排放/碳汇的影响可能为正、为负还是未知</t>
+          <t>实施气候变化减缓措施所产生、经IFCMA秘书处识别的减缓之外的其他积极成果或效益。</t>
         </is>
       </c>
       <c r="D46" s="372" t="inlineStr">
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E46" s="372" t="inlineStr">
         <is>
-          <t>正向；负向；中性；未知</t>
+          <t>适应；空气污染；能源供应安全；技术创新；减贫；就业；产业发展；其他（非穷尽清单，当前选项基于IPCC）</t>
         </is>
       </c>
       <c r="F46" s="383" t="n"/>
@@ -6812,27 +6812,15 @@
       <c r="T46" s="412" t="n"/>
     </row>
     <row r="47" ht="15" customHeight="1">
-      <c r="A47" s="282" t="n"/>
-      <c r="B47" s="371" t="inlineStr">
-        <is>
-          <t>减缓协同效益</t>
-        </is>
-      </c>
-      <c r="C47" s="371" t="inlineStr">
-        <is>
-          <t>实施气候变化减缓措施所产生、经IFCMA秘书处识别的减缓之外的其他积极成果或效益。</t>
-        </is>
-      </c>
-      <c r="D47" s="372" t="inlineStr">
-        <is>
-          <t>分类</t>
-        </is>
-      </c>
-      <c r="E47" s="372" t="inlineStr">
-        <is>
-          <t>适应；空气污染；能源供应安全；技术创新；减贫；就业；产业发展；其他（非穷尽清单，当前选项基于IPCC）</t>
-        </is>
-      </c>
+      <c r="A47" s="368" t="inlineStr">
+        <is>
+          <t>工具类型专属属性</t>
+        </is>
+      </c>
+      <c r="B47" s="261" t="n"/>
+      <c r="C47" s="261" t="n"/>
+      <c r="D47" s="261" t="n"/>
+      <c r="E47" s="262" t="n"/>
       <c r="F47" s="383" t="n"/>
       <c r="G47" s="412" t="n"/>
       <c r="H47" s="412" t="n"/>
@@ -6850,93 +6838,105 @@
       <c r="T47" s="412" t="n"/>
     </row>
     <row r="48" ht="15" customHeight="1">
-      <c r="A48" s="368" t="inlineStr">
-        <is>
-          <t>工具类型专属属性</t>
-        </is>
-      </c>
-      <c r="B48" s="261" t="n"/>
-      <c r="C48" s="261" t="n"/>
-      <c r="D48" s="261" t="n"/>
-      <c r="E48" s="262" t="n"/>
-      <c r="F48" s="383" t="n"/>
-      <c r="G48" s="412" t="n"/>
-      <c r="H48" s="412" t="n"/>
-      <c r="I48" s="412" t="n"/>
-      <c r="J48" s="412" t="n"/>
-      <c r="K48" s="412" t="n"/>
-      <c r="L48" s="412" t="n"/>
-      <c r="M48" s="412" t="n"/>
-      <c r="N48" s="412" t="n"/>
-      <c r="O48" s="412" t="n"/>
-      <c r="P48" s="412" t="n"/>
-      <c r="Q48" s="412" t="n"/>
-      <c r="R48" s="412" t="n"/>
-      <c r="S48" s="412" t="n"/>
-      <c r="T48" s="412" t="n"/>
+      <c r="A48" s="375" t="inlineStr">
+        <is>
+          <t>税收</t>
+        </is>
+      </c>
+      <c r="B48" s="380" t="inlineStr">
+        <is>
+          <t>税收及激励：年度收入</t>
+        </is>
+      </c>
+      <c r="C48" s="380" t="inlineStr">
+        <is>
+          <t>所记录税收的税收收入</t>
+        </is>
+      </c>
+      <c r="D48" s="380" t="inlineStr">
+        <is>
+          <t>数值</t>
+        </is>
+      </c>
+      <c r="E48" s="380" t="inlineStr">
+        <is>
+          <t>单位：百万本币、美元或其他适用货币</t>
+        </is>
+      </c>
+      <c r="F48" s="416" t="n"/>
+      <c r="G48" s="417" t="n"/>
+      <c r="H48" s="417" t="n"/>
+      <c r="I48" s="417" t="n"/>
+      <c r="J48" s="417" t="n"/>
+      <c r="K48" s="417" t="n"/>
+      <c r="L48" s="417" t="n"/>
+      <c r="M48" s="417" t="n"/>
+      <c r="N48" s="417" t="n"/>
+      <c r="O48" s="417" t="n"/>
+      <c r="P48" s="417" t="n"/>
+      <c r="Q48" s="417" t="n"/>
+      <c r="R48" s="417" t="n"/>
+      <c r="S48" s="417" t="n"/>
+      <c r="T48" s="417" t="n"/>
     </row>
     <row r="49" ht="15" customHeight="1">
-      <c r="A49" s="375" t="inlineStr">
-        <is>
-          <t>税收</t>
-        </is>
-      </c>
-      <c r="B49" s="380" t="inlineStr">
-        <is>
-          <t>税收及激励：年度收入</t>
-        </is>
-      </c>
-      <c r="C49" s="380" t="inlineStr">
-        <is>
-          <t>所记录税收的税收收入</t>
-        </is>
-      </c>
-      <c r="D49" s="380" t="inlineStr">
+      <c r="A49" s="293" t="n"/>
+      <c r="B49" s="372" t="inlineStr">
+        <is>
+          <t>税收及激励：专项资金</t>
+        </is>
+      </c>
+      <c r="C49" s="372" t="inlineStr">
+        <is>
+          <t>由该税收收入资助的政策（即使该政策未收录于本数据库，也在此记录）</t>
+        </is>
+      </c>
+      <c r="D49" s="372" t="inlineStr">
+        <is>
+          <t>自由文本或二元</t>
+        </is>
+      </c>
+      <c r="E49" s="372" t="inlineStr">
+        <is>
+          <t>受资助政策工具的工具ID；若受资助政策未收录于本数据库，则填“专项资金”</t>
+        </is>
+      </c>
+      <c r="F49" s="383" t="n"/>
+      <c r="G49" s="412" t="n"/>
+      <c r="H49" s="412" t="n"/>
+      <c r="I49" s="412" t="n"/>
+      <c r="J49" s="412" t="n"/>
+      <c r="K49" s="412" t="n"/>
+      <c r="L49" s="412" t="n"/>
+      <c r="M49" s="412" t="n"/>
+      <c r="N49" s="412" t="n"/>
+      <c r="O49" s="412" t="n"/>
+      <c r="P49" s="412" t="n"/>
+      <c r="Q49" s="412" t="n"/>
+      <c r="R49" s="412" t="n"/>
+      <c r="S49" s="412" t="n"/>
+      <c r="T49" s="412" t="n"/>
+    </row>
+    <row r="50" ht="15" customHeight="1">
+      <c r="A50" s="282" t="n"/>
+      <c r="B50" s="372" t="inlineStr">
+        <is>
+          <t>税收及激励：年度收入减免</t>
+        </is>
+      </c>
+      <c r="C50" s="372" t="inlineStr">
+        <is>
+          <t>若为税收优惠，填写因该税收优惠而造成的税收收入估计损失（按该工具的记录年份填写）</t>
+        </is>
+      </c>
+      <c r="D50" s="372" t="inlineStr">
         <is>
           <t>数值</t>
         </is>
       </c>
-      <c r="E49" s="380" t="inlineStr">
+      <c r="E50" s="372" t="inlineStr">
         <is>
           <t>单位：百万本币、美元或其他适用货币</t>
-        </is>
-      </c>
-      <c r="F49" s="416" t="n"/>
-      <c r="G49" s="417" t="n"/>
-      <c r="H49" s="417" t="n"/>
-      <c r="I49" s="417" t="n"/>
-      <c r="J49" s="417" t="n"/>
-      <c r="K49" s="417" t="n"/>
-      <c r="L49" s="417" t="n"/>
-      <c r="M49" s="417" t="n"/>
-      <c r="N49" s="417" t="n"/>
-      <c r="O49" s="417" t="n"/>
-      <c r="P49" s="417" t="n"/>
-      <c r="Q49" s="417" t="n"/>
-      <c r="R49" s="417" t="n"/>
-      <c r="S49" s="417" t="n"/>
-      <c r="T49" s="417" t="n"/>
-    </row>
-    <row r="50" ht="15" customHeight="1">
-      <c r="A50" s="293" t="n"/>
-      <c r="B50" s="372" t="inlineStr">
-        <is>
-          <t>税收及激励：专项资金</t>
-        </is>
-      </c>
-      <c r="C50" s="372" t="inlineStr">
-        <is>
-          <t>由该税收收入资助的政策（即使该政策未收录于本数据库，也在此记录）</t>
-        </is>
-      </c>
-      <c r="D50" s="372" t="inlineStr">
-        <is>
-          <t>自由文本或二元</t>
-        </is>
-      </c>
-      <c r="E50" s="372" t="inlineStr">
-        <is>
-          <t>受资助政策工具的工具ID；若受资助政策未收录于本数据库，则填“专项资金”</t>
         </is>
       </c>
       <c r="F50" s="383" t="n"/>
@@ -6956,15 +6956,19 @@
       <c r="T50" s="412" t="n"/>
     </row>
     <row r="51" ht="15" customHeight="1">
-      <c r="A51" s="282" t="n"/>
+      <c r="A51" s="375" t="inlineStr">
+        <is>
+          <t>补贴</t>
+        </is>
+      </c>
       <c r="B51" s="372" t="inlineStr">
         <is>
-          <t>税收及激励：年度收入减免</t>
+          <t>补贴：年度预算/支出</t>
         </is>
       </c>
       <c r="C51" s="372" t="inlineStr">
         <is>
-          <t>若为税收优惠，填写因该税收优惠而造成的税收收入估计损失（按该工具的记录年份填写）</t>
+          <t>数据收集年份之前一年安排的财政拨款或预算</t>
         </is>
       </c>
       <c r="D51" s="372" t="inlineStr">
@@ -6994,19 +6998,15 @@
       <c r="T51" s="412" t="n"/>
     </row>
     <row r="52" ht="15" customHeight="1">
-      <c r="A52" s="375" t="inlineStr">
-        <is>
-          <t>补贴</t>
-        </is>
-      </c>
+      <c r="A52" s="293" t="n"/>
       <c r="B52" s="372" t="inlineStr">
         <is>
-          <t>补贴：年度预算/支出</t>
+          <t>补贴：限额</t>
         </is>
       </c>
       <c r="C52" s="372" t="inlineStr">
         <is>
-          <t>数据收集年份之前一年安排的财政拨款或预算</t>
+          <t>该工具整个存续期内的财政拨款总额或预算总额、受补贴资产数量（容量上限）、补贴时间范围或补贴总额的其他限制</t>
         </is>
       </c>
       <c r="D52" s="372" t="inlineStr">
@@ -7016,7 +7016,7 @@
       </c>
       <c r="E52" s="372" t="inlineStr">
         <is>
-          <t>单位：百万本币、美元或其他适用货币</t>
+          <t>单位：本币、美元或其他适用货币</t>
         </is>
       </c>
       <c r="F52" s="383" t="n"/>
@@ -7039,22 +7039,22 @@
       <c r="A53" s="293" t="n"/>
       <c r="B53" s="372" t="inlineStr">
         <is>
-          <t>补贴：限额</t>
+          <t>补贴：分配机制</t>
         </is>
       </c>
       <c r="C53" s="372" t="inlineStr">
         <is>
-          <t>该工具整个存续期内的财政拨款总额或预算总额、受补贴资产数量（容量上限）、补贴时间范围或补贴总额的其他限制</t>
+          <t>补贴发放的机制</t>
         </is>
       </c>
       <c r="D53" s="372" t="inlineStr">
         <is>
-          <t>数值</t>
+          <t>分类</t>
         </is>
       </c>
       <c r="E53" s="372" t="inlineStr">
         <is>
-          <t>单位：本币、美元或其他适用货币</t>
+          <t>从清单中选择，例如：拍卖方式、默认分配、抽签等</t>
         </is>
       </c>
       <c r="F53" s="383" t="n"/>
@@ -7077,22 +7077,22 @@
       <c r="A54" s="293" t="n"/>
       <c r="B54" s="372" t="inlineStr">
         <is>
-          <t>补贴：分配机制</t>
+          <t>补贴：执行机制</t>
         </is>
       </c>
       <c r="C54" s="372" t="inlineStr">
         <is>
-          <t>补贴发放的机制</t>
+          <t>若设定了绩效要求，未达标时如何处罚</t>
         </is>
       </c>
       <c r="D54" s="372" t="inlineStr">
         <is>
-          <t>分类</t>
+          <t>分类，可补充详情</t>
         </is>
       </c>
       <c r="E54" s="372" t="inlineStr">
         <is>
-          <t>从清单中选择，例如：拍卖方式、默认分配、抽签等</t>
+          <t>行政处罚（如警告、撤销许可）；法律行动（如起诉）；罚款</t>
         </is>
       </c>
       <c r="F54" s="383" t="n"/>
@@ -7115,22 +7115,22 @@
       <c r="A55" s="293" t="n"/>
       <c r="B55" s="372" t="inlineStr">
         <is>
-          <t>补贴：执行机制</t>
+          <t>补贴：下限或上限</t>
         </is>
       </c>
       <c r="C55" s="372" t="inlineStr">
         <is>
-          <t>若设定了绩效要求，未达标时如何处罚</t>
+          <t>每年（按该工具的记录年份）补贴设定的下限或上限，指明补贴金额必须落在的区间。</t>
         </is>
       </c>
       <c r="D55" s="372" t="inlineStr">
         <is>
-          <t>分类，可补充详情</t>
+          <t>数值</t>
         </is>
       </c>
       <c r="E55" s="372" t="inlineStr">
         <is>
-          <t>行政处罚（如警告、撤销许可）；法律行动（如起诉）；罚款</t>
+          <t>以本币计</t>
         </is>
       </c>
       <c r="F55" s="383" t="n"/>
@@ -7153,22 +7153,22 @@
       <c r="A56" s="293" t="n"/>
       <c r="B56" s="372" t="inlineStr">
         <is>
-          <t>补贴：下限或上限</t>
+          <t>补贴：支持期限</t>
         </is>
       </c>
       <c r="C56" s="372" t="inlineStr">
         <is>
-          <t>每年（按该工具的记录年份）补贴设定的下限或上限，指明补贴金额必须落在的区间。</t>
+          <t>提供支持的时长（合同期限、年度付款等）</t>
         </is>
       </c>
       <c r="D56" s="372" t="inlineStr">
         <is>
-          <t>数值</t>
+          <t>自由文本</t>
         </is>
       </c>
       <c r="E56" s="372" t="inlineStr">
         <is>
-          <t>以本币计</t>
+          <t>以年或月表示</t>
         </is>
       </c>
       <c r="F56" s="383" t="n"/>
@@ -7188,27 +7188,23 @@
       <c r="T56" s="412" t="n"/>
     </row>
     <row r="57" ht="15" customHeight="1">
-      <c r="A57" s="293" t="n"/>
+      <c r="A57" s="282" t="n"/>
       <c r="B57" s="372" t="inlineStr">
         <is>
-          <t>补贴：支持期限</t>
+          <t>补贴：监测机制</t>
         </is>
       </c>
       <c r="C57" s="372" t="inlineStr">
         <is>
-          <t>提供支持的时长（合同期限、年度付款等）</t>
+          <t>任何监测方案</t>
         </is>
       </c>
       <c r="D57" s="372" t="inlineStr">
         <is>
-          <t>自由文本</t>
-        </is>
-      </c>
-      <c r="E57" s="372" t="inlineStr">
-        <is>
-          <t>以年或月表示</t>
-        </is>
-      </c>
+          <t>分类，可补充详情</t>
+        </is>
+      </c>
+      <c r="E57" s="372" t="n"/>
       <c r="F57" s="383" t="n"/>
       <c r="G57" s="412" t="n"/>
       <c r="H57" s="412" t="n"/>
@@ -7226,23 +7222,31 @@
       <c r="T57" s="412" t="n"/>
     </row>
     <row r="58" ht="15" customHeight="1">
-      <c r="A58" s="282" t="n"/>
+      <c r="A58" s="375" t="inlineStr">
+        <is>
+          <t>交易系统</t>
+        </is>
+      </c>
       <c r="B58" s="372" t="inlineStr">
         <is>
-          <t>补贴：监测机制</t>
+          <t>交易系统：类型</t>
         </is>
       </c>
       <c r="C58" s="372" t="inlineStr">
         <is>
-          <t>任何监测方案</t>
+          <t>现行交易系统，即交易配额还是信用</t>
         </is>
       </c>
       <c r="D58" s="372" t="inlineStr">
         <is>
-          <t>分类，可补充详情</t>
-        </is>
-      </c>
-      <c r="E58" s="372" t="n"/>
+          <t>分类</t>
+        </is>
+      </c>
+      <c r="E58" s="372" t="inlineStr">
+        <is>
+          <t>从清单中选择，例如：配额、信用等</t>
+        </is>
+      </c>
       <c r="F58" s="383" t="n"/>
       <c r="G58" s="412" t="n"/>
       <c r="H58" s="412" t="n"/>
@@ -7260,29 +7264,25 @@
       <c r="T58" s="412" t="n"/>
     </row>
     <row r="59" ht="15" customHeight="1">
-      <c r="A59" s="375" t="inlineStr">
-        <is>
-          <t>交易系统</t>
-        </is>
-      </c>
+      <c r="A59" s="293" t="n"/>
       <c r="B59" s="372" t="inlineStr">
         <is>
-          <t>交易系统：类型</t>
+          <t>交易系统：总量上限</t>
         </is>
       </c>
       <c r="C59" s="372" t="inlineStr">
         <is>
-          <t>现行交易系统，即交易配额还是信用</t>
+          <t>温室气体总量控制与交易或排放交易体系下，特定时期内允许的温室气体排放总量上限；若填写此格，则该工具属于配额类，否则属于信用类（与UNFCCC报告相关）</t>
         </is>
       </c>
       <c r="D59" s="372" t="inlineStr">
         <is>
-          <t>分类</t>
+          <t>自由文本</t>
         </is>
       </c>
       <c r="E59" s="372" t="inlineStr">
         <is>
-          <t>从清单中选择，例如：配额、信用等</t>
+          <t>排放交易体系填写CO2当量；若今后覆盖其他交易系统（如农业氮交易），可填写其他单位</t>
         </is>
       </c>
       <c r="F59" s="383" t="n"/>
@@ -7305,12 +7305,12 @@
       <c r="A60" s="293" t="n"/>
       <c r="B60" s="372" t="inlineStr">
         <is>
-          <t>交易系统：总量上限</t>
+          <t>交易系统：配额分配机制</t>
         </is>
       </c>
       <c r="C60" s="372" t="inlineStr">
         <is>
-          <t>温室气体总量控制与交易或排放交易体系下，特定时期内允许的温室气体排放总量上限；若填写此格，则该工具属于配额类，否则属于信用类（与UNFCCC报告相关）</t>
+          <t>交易系统内分配排放配额所采用的制度或方法，说明主体如何获得配额、配额规模以及可能的其他方面</t>
         </is>
       </c>
       <c r="D60" s="372" t="inlineStr">
@@ -7320,7 +7320,7 @@
       </c>
       <c r="E60" s="372" t="inlineStr">
         <is>
-          <t>排放交易体系填写CO2当量；若今后覆盖其他交易系统（如农业氮交易），可填写其他单位</t>
+          <t>免费配额；拍卖；两者混合</t>
         </is>
       </c>
       <c r="F60" s="383" t="n"/>
@@ -7343,22 +7343,22 @@
       <c r="A61" s="293" t="n"/>
       <c r="B61" s="372" t="inlineStr">
         <is>
-          <t>交易系统：配额分配机制</t>
+          <t>交易系统：免费配额</t>
         </is>
       </c>
       <c r="C61" s="372" t="inlineStr">
         <is>
-          <t>交易系统内分配排放配额所采用的制度或方法，说明主体如何获得配额、配额规模以及可能的其他方面</t>
+          <t>免费配额占比</t>
         </is>
       </c>
       <c r="D61" s="372" t="inlineStr">
         <is>
-          <t>自由文本</t>
+          <t>数值</t>
         </is>
       </c>
       <c r="E61" s="372" t="inlineStr">
         <is>
-          <t>免费配额；拍卖；两者混合</t>
+          <t>以百分比表示</t>
         </is>
       </c>
       <c r="F61" s="383" t="n"/>
@@ -7381,12 +7381,12 @@
       <c r="A62" s="293" t="n"/>
       <c r="B62" s="372" t="inlineStr">
         <is>
-          <t>交易系统：免费配额</t>
+          <t>交易系统：交易量</t>
         </is>
       </c>
       <c r="C62" s="372" t="inlineStr">
         <is>
-          <t>免费配额占比</t>
+          <t>收集年份前一年的交易量</t>
         </is>
       </c>
       <c r="D62" s="372" t="inlineStr">
@@ -7396,7 +7396,7 @@
       </c>
       <c r="E62" s="372" t="inlineStr">
         <is>
-          <t>以百分比表示</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="F62" s="383" t="n"/>
@@ -7419,22 +7419,22 @@
       <c r="A63" s="293" t="n"/>
       <c r="B63" s="372" t="inlineStr">
         <is>
-          <t>交易系统：交易量</t>
+          <t>交易系统：链接</t>
         </is>
       </c>
       <c r="C63" s="372" t="inlineStr">
         <is>
-          <t>收集年份前一年的交易量</t>
+          <t>与其他排放交易体系的链接</t>
         </is>
       </c>
       <c r="D63" s="372" t="inlineStr">
         <is>
-          <t>数值</t>
+          <t>自由文本</t>
         </is>
       </c>
       <c r="E63" s="372" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>填写相关工具的工具ID（无链接填N/A）</t>
         </is>
       </c>
       <c r="F63" s="383" t="n"/>
@@ -7457,22 +7457,22 @@
       <c r="A64" s="293" t="n"/>
       <c r="B64" s="372" t="inlineStr">
         <is>
-          <t>交易系统：链接</t>
+          <t>交易系统：市场稳定机制</t>
         </is>
       </c>
       <c r="C64" s="372" t="inlineStr">
         <is>
-          <t>与其他排放交易体系的链接</t>
+          <t>交易系统内是否存在任何旨在稳定市场、防止价格剧烈波动或应对供需失衡的机制或安排。例如：二级市场/抵消与信用</t>
         </is>
       </c>
       <c r="D64" s="372" t="inlineStr">
         <is>
-          <t>自由文本</t>
+          <t>二元，可补充详情</t>
         </is>
       </c>
       <c r="E64" s="372" t="inlineStr">
         <is>
-          <t>填写相关工具的工具ID（无链接填N/A）</t>
+          <t>是/否</t>
         </is>
       </c>
       <c r="F64" s="383" t="n"/>
@@ -7495,22 +7495,22 @@
       <c r="A65" s="293" t="n"/>
       <c r="B65" s="372" t="inlineStr">
         <is>
-          <t>交易系统：市场稳定机制</t>
+          <t>交易系统：年收入</t>
         </is>
       </c>
       <c r="C65" s="372" t="inlineStr">
         <is>
-          <t>交易系统内是否存在任何旨在稳定市场、防止价格剧烈波动或应对供需失衡的机制或安排。例如：二级市场/抵消与信用</t>
+          <t>交易系统每年产生的收入，包括与排放交易相关的各类费用、罚款或其他资金流（指系统收入，而非政府收入）</t>
         </is>
       </c>
       <c r="D65" s="372" t="inlineStr">
         <is>
-          <t>二元，可补充详情</t>
+          <t>自由文本</t>
         </is>
       </c>
       <c r="E65" s="372" t="inlineStr">
         <is>
-          <t>是/否</t>
+          <t>以本币计（收集年份前一年）</t>
         </is>
       </c>
       <c r="F65" s="383" t="n"/>
@@ -7533,12 +7533,12 @@
       <c r="A66" s="293" t="n"/>
       <c r="B66" s="372" t="inlineStr">
         <is>
-          <t>交易系统：年收入</t>
+          <t>交易系统：允许使用抵消</t>
         </is>
       </c>
       <c r="C66" s="372" t="inlineStr">
         <is>
-          <t>交易系统每年产生的收入，包括与排放交易相关的各类费用、罚款或其他资金流（指系统收入，而非政府收入）</t>
+          <t>允许使用何种抵消的规则或对相关规则的引用；若不允许使用抵消，则填“否”</t>
         </is>
       </c>
       <c r="D66" s="372" t="inlineStr">
@@ -7548,7 +7548,7 @@
       </c>
       <c r="E66" s="372" t="inlineStr">
         <is>
-          <t>以本币计（收集年份前一年）</t>
+          <t>无则填“否”；否则描述适用规则</t>
         </is>
       </c>
       <c r="F66" s="383" t="n"/>
@@ -7568,25 +7568,25 @@
       <c r="T66" s="412" t="n"/>
     </row>
     <row r="67" ht="15" customHeight="1">
-      <c r="A67" s="293" t="n"/>
+      <c r="A67" s="282" t="n"/>
       <c r="B67" s="372" t="inlineStr">
         <is>
-          <t>交易系统：允许使用抵消</t>
+          <t>交易系统：违规处罚</t>
         </is>
       </c>
       <c r="C67" s="372" t="inlineStr">
         <is>
-          <t>允许使用何种抵消的规则或对相关规则的引用；若不允许使用抵消，则填“否”</t>
+          <t>对未遵守排放交易体系规定和要求的主体施加的后果或罚款</t>
         </is>
       </c>
       <c r="D67" s="372" t="inlineStr">
         <is>
-          <t>自由文本</t>
+          <t>分类，可补充详情</t>
         </is>
       </c>
       <c r="E67" s="372" t="inlineStr">
         <is>
-          <t>无则填“否”；否则描述适用规则</t>
+          <t>行政处罚（如警告、撤销许可）；法律行动（如起诉）；罚款</t>
         </is>
       </c>
       <c r="F67" s="383" t="n"/>
@@ -7606,25 +7606,29 @@
       <c r="T67" s="412" t="n"/>
     </row>
     <row r="68" ht="15" customHeight="1">
-      <c r="A68" s="282" t="n"/>
-      <c r="B68" s="372" t="inlineStr">
-        <is>
-          <t>交易系统：违规处罚</t>
-        </is>
-      </c>
-      <c r="C68" s="372" t="inlineStr">
-        <is>
-          <t>对未遵守排放交易体系规定和要求的主体施加的后果或罚款</t>
-        </is>
-      </c>
-      <c r="D68" s="372" t="inlineStr">
-        <is>
-          <t>分类，可补充详情</t>
-        </is>
-      </c>
-      <c r="E68" s="372" t="inlineStr">
-        <is>
-          <t>行政处罚（如警告、撤销许可）；法律行动（如起诉）；罚款</t>
+      <c r="A68" s="375" t="inlineStr">
+        <is>
+          <t>规制工具</t>
+        </is>
+      </c>
+      <c r="B68" s="371" t="inlineStr">
+        <is>
+          <t>合规监测</t>
+        </is>
+      </c>
+      <c r="C68" s="371" t="inlineStr">
+        <is>
+          <t>记录是否设有监测和确保气候变化减缓政策合规性的方法、流程或制度</t>
+        </is>
+      </c>
+      <c r="D68" s="371" t="inlineStr">
+        <is>
+          <t>分类（单选），可补充详情</t>
+        </is>
+      </c>
+      <c r="E68" s="371" t="inlineStr">
+        <is>
+          <t>无合规监测；自我监测与报告；政府主管部门或第三方开展的检查或审计；其他</t>
         </is>
       </c>
       <c r="F68" s="383" t="n"/>
@@ -7644,29 +7648,25 @@
       <c r="T68" s="412" t="n"/>
     </row>
     <row r="69" ht="15" customHeight="1">
-      <c r="A69" s="375" t="inlineStr">
-        <is>
-          <t>规制工具</t>
-        </is>
-      </c>
+      <c r="A69" s="293" t="n"/>
       <c r="B69" s="371" t="inlineStr">
         <is>
-          <t>合规监测</t>
+          <t>合规监测详情</t>
         </is>
       </c>
       <c r="C69" s="371" t="inlineStr">
         <is>
-          <t>记录是否设有监测和确保气候变化减缓政策合规性的方法、流程或制度</t>
+          <t>记录合规监测方式的具体情况（即自我监测与报告；政府主管部门或第三方开展的检查或审计；其他）</t>
         </is>
       </c>
       <c r="D69" s="371" t="inlineStr">
         <is>
-          <t>分类（单选），可补充详情</t>
+          <t>自由文本</t>
         </is>
       </c>
       <c r="E69" s="371" t="inlineStr">
         <is>
-          <t>无合规监测；自我监测与报告；政府主管部门或第三方开展的检查或审计；其他</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="F69" s="383" t="n"/>
@@ -7689,22 +7689,22 @@
       <c r="A70" s="293" t="n"/>
       <c r="B70" s="371" t="inlineStr">
         <is>
-          <t>合规监测详情</t>
+          <t>合规执行</t>
         </is>
       </c>
       <c r="C70" s="371" t="inlineStr">
         <is>
-          <t>记录合规监测方式的具体情况（即自我监测与报告；政府主管部门或第三方开展的检查或审计；其他）</t>
+          <t>对未遵守气候变化减缓政策规制要求的主体施加的后果</t>
         </is>
       </c>
       <c r="D70" s="371" t="inlineStr">
         <is>
-          <t>自由文本</t>
+          <t>分类（多选），可补充详情</t>
         </is>
       </c>
       <c r="E70" s="371" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>无合规执行；罚款；禁止；合规命令；其他</t>
         </is>
       </c>
       <c r="F70" s="383" t="n"/>
@@ -7727,22 +7727,22 @@
       <c r="A71" s="293" t="n"/>
       <c r="B71" s="371" t="inlineStr">
         <is>
-          <t>合规执行</t>
+          <t>合规执行详情</t>
         </is>
       </c>
       <c r="C71" s="371" t="inlineStr">
         <is>
-          <t>对未遵守气候变化减缓政策规制要求的主体施加的后果</t>
+          <t>记录执行方式和流程的具体情况（即罚款；禁止；合规命令；其他）</t>
         </is>
       </c>
       <c r="D71" s="371" t="inlineStr">
         <is>
-          <t>分类（多选），可补充详情</t>
+          <t>自由文本</t>
         </is>
       </c>
       <c r="E71" s="371" t="inlineStr">
         <is>
-          <t>无合规执行；罚款；禁止；合规命令；其他</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="F71" s="383" t="n"/>
@@ -7765,22 +7765,22 @@
       <c r="A72" s="293" t="n"/>
       <c r="B72" s="371" t="inlineStr">
         <is>
-          <t>合规执行详情</t>
+          <t>合规促进</t>
         </is>
       </c>
       <c r="C72" s="371" t="inlineStr">
         <is>
-          <t>记录执行方式和流程的具体情况（即罚款；禁止；合规命令；其他）</t>
+          <t>旨在鼓励和促进遵守气候变化减缓政策规制措施的举措或活动</t>
         </is>
       </c>
       <c r="D72" s="371" t="inlineStr">
         <is>
-          <t>自由文本</t>
+          <t>分类（多选），可补充详情</t>
         </is>
       </c>
       <c r="E72" s="371" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>无合规促进；规制激励（如加权、储存、汇集、交易）；信息与直接协助；资金支持；其他激励或支持</t>
         </is>
       </c>
       <c r="F72" s="383" t="n"/>
@@ -7800,25 +7800,25 @@
       <c r="T72" s="412" t="n"/>
     </row>
     <row r="73" ht="15" customHeight="1">
-      <c r="A73" s="293" t="n"/>
+      <c r="A73" s="282" t="n"/>
       <c r="B73" s="371" t="inlineStr">
         <is>
-          <t>合规促进</t>
+          <t>合规促进详情</t>
         </is>
       </c>
       <c r="C73" s="371" t="inlineStr">
         <is>
-          <t>旨在鼓励和促进遵守气候变化减缓政策规制措施的举措或活动</t>
+          <t>记录合规促进方式和流程的具体情况（例如规制激励如加权、储存、汇集、交易等的详情；信息/直接协助；资金支持；其他合规促进流程）</t>
         </is>
       </c>
       <c r="D73" s="371" t="inlineStr">
         <is>
-          <t>分类（多选），可补充详情</t>
+          <t>自由文本</t>
         </is>
       </c>
       <c r="E73" s="371" t="inlineStr">
         <is>
-          <t>无合规促进；规制激励（如加权、储存、汇集、交易）；信息与直接协助；资金支持；其他激励或支持</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="F73" s="383" t="n"/>
@@ -7838,25 +7838,29 @@
       <c r="T73" s="412" t="n"/>
     </row>
     <row r="74" ht="15" customHeight="1">
-      <c r="A74" s="282" t="n"/>
+      <c r="A74" s="375" t="inlineStr">
+        <is>
+          <t>政府投资与消费</t>
+        </is>
+      </c>
       <c r="B74" s="371" t="inlineStr">
         <is>
-          <t>合规促进详情</t>
+          <t>公共投资：共同融资</t>
         </is>
       </c>
       <c r="C74" s="371" t="inlineStr">
         <is>
-          <t>记录合规促进方式和流程的具体情况（例如规制激励如加权、储存、汇集、交易等的详情；信息/直接协助；资金支持；其他合规促进流程）</t>
+          <t>指明政府是全额资助该项目/技术，还是与其他方共同出资</t>
         </is>
       </c>
       <c r="D74" s="371" t="inlineStr">
         <is>
-          <t>自由文本</t>
+          <t>分类（单选）</t>
         </is>
       </c>
       <c r="E74" s="371" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>是；否</t>
         </is>
       </c>
       <c r="F74" s="383" t="n"/>
@@ -7876,24 +7880,20 @@
       <c r="T74" s="412" t="n"/>
     </row>
     <row r="75" ht="15" customHeight="1">
-      <c r="A75" s="375" t="inlineStr">
-        <is>
-          <t>政府投资与消费</t>
-        </is>
-      </c>
+      <c r="A75" s="293" t="n"/>
       <c r="B75" s="371" t="inlineStr">
         <is>
-          <t>公共投资：共同融资</t>
+          <t>公共投资：选择流程</t>
         </is>
       </c>
       <c r="C75" s="371" t="inlineStr">
         <is>
-          <t>指明政府是全额资助该项目/技术，还是与其他方共同出资</t>
+          <t>项目或投资如何被选定为投资对象的相关详情。若存在规范的遴选流程，填写遴选标准</t>
         </is>
       </c>
       <c r="D75" s="371" t="inlineStr">
         <is>
-          <t>分类（单选）</t>
+          <t>分类（单选），可补充详情</t>
         </is>
       </c>
       <c r="E75" s="371" t="inlineStr">
@@ -7921,12 +7921,12 @@
       <c r="A76" s="293" t="n"/>
       <c r="B76" s="371" t="inlineStr">
         <is>
-          <t>公共投资：选择流程</t>
+          <t>公共采购：招标流程</t>
         </is>
       </c>
       <c r="C76" s="371" t="inlineStr">
         <is>
-          <t>项目或投资如何被选定为投资对象的相关详情。若存在规范的遴选流程，填写遴选标准</t>
+          <t>指明招标/采购流程的类型</t>
         </is>
       </c>
       <c r="D76" s="371" t="inlineStr">
@@ -7936,7 +7936,7 @@
       </c>
       <c r="E76" s="371" t="inlineStr">
         <is>
-          <t>是；否</t>
+          <t>公开招标；直接采购；议价采购；加速公开招标</t>
         </is>
       </c>
       <c r="F76" s="383" t="n"/>
@@ -7959,22 +7959,22 @@
       <c r="A77" s="293" t="n"/>
       <c r="B77" s="371" t="inlineStr">
         <is>
-          <t>公共采购：招标流程</t>
+          <t>公共采购：招标评标标准</t>
         </is>
       </c>
       <c r="C77" s="371" t="inlineStr">
         <is>
-          <t>指明招标/采购流程的类型</t>
+          <t>指明招标过程中是否对满足特定要求的投标人给予加分或优待</t>
         </is>
       </c>
       <c r="D77" s="371" t="inlineStr">
         <is>
-          <t>分类（单选），可补充详情</t>
+          <t>自由文本</t>
         </is>
       </c>
       <c r="E77" s="371" t="inlineStr">
         <is>
-          <t>公开招标；直接采购；议价采购；加速公开招标</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="F77" s="383" t="n"/>
@@ -7997,22 +7997,22 @@
       <c r="A78" s="293" t="n"/>
       <c r="B78" s="371" t="inlineStr">
         <is>
-          <t>公共采购：招标评标标准</t>
+          <t>公共采购：合规监测</t>
         </is>
       </c>
       <c r="C78" s="371" t="inlineStr">
         <is>
-          <t>指明招标过程中是否对满足特定要求的投标人给予加分或优待</t>
+          <t>监测和确保气候变化减缓政策合规性的现行方法、流程或制度</t>
         </is>
       </c>
       <c r="D78" s="371" t="inlineStr">
         <is>
-          <t>自由文本</t>
+          <t>分类（单选），可补充详情</t>
         </is>
       </c>
       <c r="E78" s="371" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>无合规监测；自我监测与报告；政府主管部门或第三方开展的检查或审计；其他</t>
         </is>
       </c>
       <c r="F78" s="383" t="n"/>
@@ -8035,22 +8035,22 @@
       <c r="A79" s="293" t="n"/>
       <c r="B79" s="371" t="inlineStr">
         <is>
-          <t>公共采购：合规监测</t>
+          <t>公共采购：合规执行</t>
         </is>
       </c>
       <c r="C79" s="371" t="inlineStr">
         <is>
-          <t>监测和确保气候变化减缓政策合规性的现行方法、流程或制度</t>
+          <t>对未遵守气候变化减缓政策规制要求的主体施加的后果</t>
         </is>
       </c>
       <c r="D79" s="371" t="inlineStr">
         <is>
-          <t>分类（单选），可补充详情</t>
+          <t>分类（多选），可补充详情</t>
         </is>
       </c>
       <c r="E79" s="371" t="inlineStr">
         <is>
-          <t>无合规监测；自我监测与报告；政府主管部门或第三方开展的检查或审计；其他</t>
+          <t>无合规执行；罚款；禁止；合规命令；其他</t>
         </is>
       </c>
       <c r="F79" s="383" t="n"/>
@@ -8073,22 +8073,22 @@
       <c r="A80" s="293" t="n"/>
       <c r="B80" s="371" t="inlineStr">
         <is>
-          <t>公共采购：合规执行</t>
+          <t>公共采购：全生命周期成本</t>
         </is>
       </c>
       <c r="C80" s="371" t="inlineStr">
         <is>
-          <t>对未遵守气候变化减缓政策规制要求的主体施加的后果</t>
+          <t>在评估财务方案时考虑产品、服务或工程全生命周期的总成本，包括：（i）采购价格及所有相关成本（运输、安装、保险等）；（ii）运行成本，包括能源、燃料和水的使用、备件与维护；（iii）生命周期末期成本，如退役或处置；以及（iv）计入环境外部性的成本。</t>
         </is>
       </c>
       <c r="D80" s="371" t="inlineStr">
         <is>
-          <t>分类（多选），可补充详情</t>
+          <t>分类（单选）</t>
         </is>
       </c>
       <c r="E80" s="371" t="inlineStr">
         <is>
-          <t>无合规执行；罚款；禁止；合规命令；其他</t>
+          <t>是；否</t>
         </is>
       </c>
       <c r="F80" s="383" t="n"/>
@@ -8108,25 +8108,25 @@
       <c r="T80" s="412" t="n"/>
     </row>
     <row r="81" ht="15" customHeight="1">
-      <c r="A81" s="293" t="n"/>
-      <c r="B81" s="371" t="inlineStr">
-        <is>
-          <t>公共采购：全生命周期成本</t>
-        </is>
-      </c>
-      <c r="C81" s="371" t="inlineStr">
-        <is>
-          <t>在评估财务方案时考虑产品、服务或工程全生命周期的总成本，包括：（i）采购价格及所有相关成本（运输、安装、保险等）；（ii）运行成本，包括能源、燃料和水的使用、备件与维护；（iii）生命周期末期成本，如退役或处置；以及（iv）计入环境外部性的成本。</t>
-        </is>
-      </c>
-      <c r="D81" s="371" t="inlineStr">
-        <is>
-          <t>分类（单选）</t>
-        </is>
-      </c>
-      <c r="E81" s="371" t="inlineStr">
-        <is>
-          <t>是；否</t>
+      <c r="A81" s="282" t="n"/>
+      <c r="B81" s="372" t="inlineStr">
+        <is>
+          <t>公共投资/采购：年度支出</t>
+        </is>
+      </c>
+      <c r="C81" s="372" t="inlineStr">
+        <is>
+          <t>数据收集年份之前一年安排的财政拨款或预算</t>
+        </is>
+      </c>
+      <c r="D81" s="372" t="inlineStr">
+        <is>
+          <t>数值</t>
+        </is>
+      </c>
+      <c r="E81" s="372" t="inlineStr">
+        <is>
+          <t>单位：百万本币、美元或其他适用货币</t>
         </is>
       </c>
       <c r="F81" s="383" t="n"/>
@@ -8146,25 +8146,29 @@
       <c r="T81" s="412" t="n"/>
     </row>
     <row r="82" ht="15" customHeight="1">
-      <c r="A82" s="282" t="n"/>
-      <c r="B82" s="372" t="inlineStr">
-        <is>
-          <t>公共投资/采购：年度支出</t>
-        </is>
-      </c>
-      <c r="C82" s="372" t="inlineStr">
-        <is>
-          <t>数据收集年份之前一年安排的财政拨款或预算</t>
-        </is>
-      </c>
-      <c r="D82" s="372" t="inlineStr">
-        <is>
-          <t>数值</t>
-        </is>
-      </c>
-      <c r="E82" s="372" t="inlineStr">
-        <is>
-          <t>单位：百万本币、美元或其他适用货币</t>
+      <c r="A82" s="375" t="inlineStr">
+        <is>
+          <t>信息工具</t>
+        </is>
+      </c>
+      <c r="B82" s="371" t="inlineStr">
+        <is>
+          <t>工具联动</t>
+        </is>
+      </c>
+      <c r="C82" s="371" t="inlineStr">
+        <is>
+          <t>记录该信息工具是否与其他工具直接联动</t>
+        </is>
+      </c>
+      <c r="D82" s="371" t="inlineStr">
+        <is>
+          <t>自由文本</t>
+        </is>
+      </c>
+      <c r="E82" s="371" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="F82" s="383" t="n"/>
@@ -8184,29 +8188,25 @@
       <c r="T82" s="412" t="n"/>
     </row>
     <row r="83" ht="15" customHeight="1">
-      <c r="A83" s="375" t="inlineStr">
-        <is>
-          <t>信息工具</t>
-        </is>
-      </c>
+      <c r="A83" s="293" t="n"/>
       <c r="B83" s="371" t="inlineStr">
         <is>
-          <t>工具联动</t>
+          <t>信息采集责任方</t>
         </is>
       </c>
       <c r="C83" s="371" t="inlineStr">
         <is>
-          <t>记录该信息工具是否与其他工具直接联动</t>
+          <t>负责采集所需信息的主体详情</t>
         </is>
       </c>
       <c r="D83" s="371" t="inlineStr">
         <is>
-          <t>自由文本</t>
+          <t>分类（单选）</t>
         </is>
       </c>
       <c r="E83" s="371" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>政府主管部门（检查或审计）；第三方（检查或审计）；受规制主体（自行报告）</t>
         </is>
       </c>
       <c r="F83" s="383" t="n"/>
@@ -8229,22 +8229,22 @@
       <c r="A84" s="293" t="n"/>
       <c r="B84" s="371" t="inlineStr">
         <is>
-          <t>信息采集责任方</t>
+          <t>信息传输方式</t>
         </is>
       </c>
       <c r="C84" s="371" t="inlineStr">
         <is>
-          <t>负责采集所需信息的主体详情</t>
+          <t>指明信息以何种方式传递给政府</t>
         </is>
       </c>
       <c r="D84" s="371" t="inlineStr">
         <is>
-          <t>分类（单选）</t>
+          <t>自由文本</t>
         </is>
       </c>
       <c r="E84" s="371" t="inlineStr">
         <is>
-          <t>政府主管部门（检查或审计）；第三方（检查或审计）；受规制主体（自行报告）</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="F84" s="383" t="n"/>
@@ -8267,22 +8267,22 @@
       <c r="A85" s="293" t="n"/>
       <c r="B85" s="371" t="inlineStr">
         <is>
-          <t>信息传输方式</t>
+          <t>信息提供频率</t>
         </is>
       </c>
       <c r="C85" s="371" t="inlineStr">
         <is>
-          <t>指明信息以何种方式传递给政府</t>
+          <t>指明信息须以何种频率提供</t>
         </is>
       </c>
       <c r="D85" s="371" t="inlineStr">
         <is>
-          <t>自由文本</t>
+          <t>分类（单选），可补充详情</t>
         </is>
       </c>
       <c r="E85" s="371" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>实时；每季度；每年；其他，详情：__</t>
         </is>
       </c>
       <c r="F85" s="383" t="n"/>
@@ -8305,22 +8305,22 @@
       <c r="A86" s="293" t="n"/>
       <c r="B86" s="371" t="inlineStr">
         <is>
-          <t>信息提供频率</t>
+          <t>信息公开可用性</t>
         </is>
       </c>
       <c r="C86" s="371" t="inlineStr">
         <is>
-          <t>指明信息须以何种频率提供</t>
+          <t>信息是否公开可得，以及若公开，可通过何种渠道获取</t>
         </is>
       </c>
       <c r="D86" s="371" t="inlineStr">
         <is>
-          <t>分类（单选），可补充详情</t>
+          <t>自由文本</t>
         </is>
       </c>
       <c r="E86" s="371" t="inlineStr">
         <is>
-          <t>实时；每季度；每年；其他，详情：__</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="F86" s="383" t="n"/>
@@ -8343,22 +8343,22 @@
       <c r="A87" s="293" t="n"/>
       <c r="B87" s="371" t="inlineStr">
         <is>
-          <t>信息公开可用性</t>
+          <t>标签类型</t>
         </is>
       </c>
       <c r="C87" s="371" t="inlineStr">
         <is>
-          <t>信息是否公开可得，以及若公开，可通过何种渠道获取</t>
+          <t>指明标签的授予和设计方式</t>
         </is>
       </c>
       <c r="D87" s="371" t="inlineStr">
         <is>
-          <t>自由文本</t>
+          <t>分类</t>
         </is>
       </c>
       <c r="E87" s="371" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>二元（基于单一阈值）；分类；连续</t>
         </is>
       </c>
       <c r="F87" s="383" t="n"/>
@@ -8381,22 +8381,22 @@
       <c r="A88" s="293" t="n"/>
       <c r="B88" s="371" t="inlineStr">
         <is>
-          <t>标签类型</t>
+          <t>合规监测</t>
         </is>
       </c>
       <c r="C88" s="371" t="inlineStr">
         <is>
-          <t>指明标签的授予和设计方式</t>
+          <t>监测和确保气候变化减缓政策合规性的现行方法、流程或制度</t>
         </is>
       </c>
       <c r="D88" s="371" t="inlineStr">
         <is>
-          <t>分类</t>
+          <t>分类（单选），可补充详情</t>
         </is>
       </c>
       <c r="E88" s="371" t="inlineStr">
         <is>
-          <t>二元（基于单一阈值）；分类；连续</t>
+          <t>无合规监测；随机；按标准定向：__；固定时间间隔：__；不定期；事先通知的检查/审计；不事先通知的检查/审计</t>
         </is>
       </c>
       <c r="F88" s="383" t="n"/>
@@ -8419,22 +8419,22 @@
       <c r="A89" s="293" t="n"/>
       <c r="B89" s="371" t="inlineStr">
         <is>
-          <t>合规监测</t>
+          <t>合规执行</t>
         </is>
       </c>
       <c r="C89" s="371" t="inlineStr">
         <is>
-          <t>监测和确保气候变化减缓政策合规性的现行方法、流程或制度</t>
+          <t>对未遵守气候变化减缓政策规制要求的主体施加的后果</t>
         </is>
       </c>
       <c r="D89" s="371" t="inlineStr">
         <is>
-          <t>分类（单选），可补充详情</t>
+          <t>分类（多选），可补充详情</t>
         </is>
       </c>
       <c r="E89" s="371" t="inlineStr">
         <is>
-          <t>无合规监测；随机；按标准定向：__；固定时间间隔：__；不定期；事先通知的检查/审计；不事先通知的检查/审计</t>
+          <t>无合规执行；罚款；禁止；合规命令；其他</t>
         </is>
       </c>
       <c r="F89" s="383" t="n"/>
@@ -8457,12 +8457,12 @@
       <c r="A90" s="293" t="n"/>
       <c r="B90" s="371" t="inlineStr">
         <is>
-          <t>合规执行</t>
+          <t>合规促进</t>
         </is>
       </c>
       <c r="C90" s="371" t="inlineStr">
         <is>
-          <t>对未遵守气候变化减缓政策规制要求的主体施加的后果</t>
+          <t>旨在鼓励和促进遵守气候变化减缓政策规制措施的举措或活动</t>
         </is>
       </c>
       <c r="D90" s="371" t="inlineStr">
@@ -8472,7 +8472,7 @@
       </c>
       <c r="E90" s="371" t="inlineStr">
         <is>
-          <t>无合规执行；罚款；禁止；合规命令；其他</t>
+          <t>无合规促进；信息与直接协助；资金支持；其他激励或支持</t>
         </is>
       </c>
       <c r="F90" s="383" t="n"/>
@@ -8492,25 +8492,25 @@
       <c r="T90" s="412" t="n"/>
     </row>
     <row r="91" ht="15" customHeight="1">
-      <c r="A91" s="293" t="n"/>
+      <c r="A91" s="282" t="n"/>
       <c r="B91" s="371" t="inlineStr">
         <is>
-          <t>合规促进</t>
+          <t>能力建设、培训/教育、宣传和奖励计划详情</t>
         </is>
       </c>
       <c r="C91" s="371" t="inlineStr">
         <is>
-          <t>旨在鼓励和促进遵守气候变化减缓政策规制措施的举措或活动</t>
+          <t>填写频率、目标群体和年度预算安排的详情</t>
         </is>
       </c>
       <c r="D91" s="371" t="inlineStr">
         <is>
-          <t>分类（多选），可补充详情</t>
+          <t>自由文本</t>
         </is>
       </c>
       <c r="E91" s="371" t="inlineStr">
         <is>
-          <t>无合规促进；信息与直接协助；资金支持；其他激励或支持</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="F91" s="383" t="n"/>
@@ -8530,25 +8530,29 @@
       <c r="T91" s="412" t="n"/>
     </row>
     <row r="92" ht="15" customHeight="1">
-      <c r="A92" s="282" t="n"/>
-      <c r="B92" s="371" t="inlineStr">
-        <is>
-          <t>能力建设、培训/教育、宣传和奖励计划详情</t>
-        </is>
-      </c>
-      <c r="C92" s="371" t="inlineStr">
-        <is>
-          <t>填写频率、目标群体和年度预算安排的详情</t>
-        </is>
-      </c>
-      <c r="D92" s="371" t="inlineStr">
-        <is>
-          <t>自由文本</t>
-        </is>
-      </c>
-      <c r="E92" s="371" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="A92" s="375" t="inlineStr">
+        <is>
+          <t>自愿措施</t>
+        </is>
+      </c>
+      <c r="B92" s="372" t="inlineStr">
+        <is>
+          <t>参与激励</t>
+        </is>
+      </c>
+      <c r="C92" s="372" t="inlineStr">
+        <is>
+          <t>为鼓励自愿参与气候变化减缓活动或项目而提供的奖励、利益或正向激励</t>
+        </is>
+      </c>
+      <c r="D92" s="372" t="inlineStr">
+        <is>
+          <t>分类（单选）</t>
+        </is>
+      </c>
+      <c r="E92" s="372" t="inlineStr">
+        <is>
+          <t>资金性；规制性；声誉性；无</t>
         </is>
       </c>
       <c r="F92" s="383" t="n"/>
@@ -8568,29 +8572,25 @@
       <c r="T92" s="412" t="n"/>
     </row>
     <row r="93" ht="15" customHeight="1">
-      <c r="A93" s="375" t="inlineStr">
-        <is>
-          <t>自愿措施</t>
-        </is>
-      </c>
+      <c r="A93" s="293" t="n"/>
       <c r="B93" s="372" t="inlineStr">
         <is>
-          <t>参与激励</t>
+          <t>监测</t>
         </is>
       </c>
       <c r="C93" s="372" t="inlineStr">
         <is>
-          <t>为鼓励自愿参与气候变化减缓活动或项目而提供的奖励、利益或正向激励</t>
+          <t>跟踪和评估气候变化减缓相关自愿行动或倡议的现行流程和制度</t>
         </is>
       </c>
       <c r="D93" s="372" t="inlineStr">
         <is>
-          <t>分类（单选）</t>
+          <t>二元，可补充详情</t>
         </is>
       </c>
       <c r="E93" s="372" t="inlineStr">
         <is>
-          <t>资金性；规制性；声誉性；无</t>
+          <t>是/否，可补充详情</t>
         </is>
       </c>
       <c r="F93" s="383" t="n"/>
@@ -8609,16 +8609,16 @@
       <c r="S93" s="412" t="n"/>
       <c r="T93" s="412" t="n"/>
     </row>
-    <row r="94" ht="15" customHeight="1">
-      <c r="A94" s="293" t="n"/>
+    <row r="94">
+      <c r="A94" s="282" t="n"/>
       <c r="B94" s="372" t="inlineStr">
         <is>
-          <t>监测</t>
+          <t>违规制裁</t>
         </is>
       </c>
       <c r="C94" s="372" t="inlineStr">
         <is>
-          <t>跟踪和评估气候变化减缓相关自愿行动或倡议的现行流程和制度</t>
+          <t>对未能履行气候变化减缓相关自愿承诺或义务的主体或个人施加的后果或处罚</t>
         </is>
       </c>
       <c r="D94" s="372" t="inlineStr">
@@ -8647,61 +8647,24 @@
       <c r="S94" s="412" t="n"/>
       <c r="T94" s="412" t="n"/>
     </row>
-    <row r="95" ht="15" customHeight="1">
-      <c r="A95" s="282" t="n"/>
-      <c r="B95" s="372" t="inlineStr">
-        <is>
-          <t>违规制裁</t>
-        </is>
-      </c>
-      <c r="C95" s="372" t="inlineStr">
-        <is>
-          <t>对未能履行气候变化减缓相关自愿承诺或义务的主体或个人施加的后果或处罚</t>
-        </is>
-      </c>
-      <c r="D95" s="372" t="inlineStr">
-        <is>
-          <t>二元，可补充详情</t>
-        </is>
-      </c>
-      <c r="E95" s="372" t="inlineStr">
-        <is>
-          <t>是/否，可补充详情</t>
-        </is>
-      </c>
-      <c r="F95" s="383" t="n"/>
-      <c r="G95" s="412" t="n"/>
-      <c r="H95" s="412" t="n"/>
-      <c r="I95" s="412" t="n"/>
-      <c r="J95" s="412" t="n"/>
-      <c r="K95" s="412" t="n"/>
-      <c r="L95" s="412" t="n"/>
-      <c r="M95" s="412" t="n"/>
-      <c r="N95" s="412" t="n"/>
-      <c r="O95" s="412" t="n"/>
-      <c r="P95" s="412" t="n"/>
-      <c r="Q95" s="412" t="n"/>
-      <c r="R95" s="412" t="n"/>
-      <c r="S95" s="412" t="n"/>
-      <c r="T95" s="412" t="n"/>
-    </row>
+    <row r="95" ht="15" customHeight="1"/>
   </sheetData>
   <mergeCells count="15">
     <mergeCell ref="A4:A7"/>
-    <mergeCell ref="A39:A41"/>
-    <mergeCell ref="A44:A47"/>
-    <mergeCell ref="A75:A82"/>
-    <mergeCell ref="A48:E48"/>
-    <mergeCell ref="A52:A58"/>
+    <mergeCell ref="A23:A37"/>
+    <mergeCell ref="A48:A50"/>
+    <mergeCell ref="A74:A81"/>
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A42:A43"/>
-    <mergeCell ref="A69:A74"/>
-    <mergeCell ref="A8:A23"/>
-    <mergeCell ref="A83:A92"/>
-    <mergeCell ref="A59:A68"/>
-    <mergeCell ref="A24:A38"/>
-    <mergeCell ref="A93:A95"/>
-    <mergeCell ref="A49:A51"/>
+    <mergeCell ref="A43:A46"/>
+    <mergeCell ref="A51:A57"/>
+    <mergeCell ref="A92:A94"/>
+    <mergeCell ref="A82:A91"/>
+    <mergeCell ref="A47:E47"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="A38:A40"/>
+    <mergeCell ref="A68:A73"/>
+    <mergeCell ref="A8:A22"/>
+    <mergeCell ref="A58:A67"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9196,7 +9159,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BN2"/>
+  <dimension ref="A1:BM2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
@@ -9228,12 +9191,12 @@
       <c r="S1" s="325" t="n"/>
       <c r="T1" s="325" t="n"/>
       <c r="U1" s="325" t="n"/>
-      <c r="V1" s="325" t="n"/>
-      <c r="W1" s="326" t="inlineStr">
+      <c r="V1" s="326" t="inlineStr">
         <is>
           <t>政策规制基础与强度</t>
         </is>
       </c>
+      <c r="W1" s="327" t="n"/>
       <c r="X1" s="327" t="n"/>
       <c r="Y1" s="327" t="n"/>
       <c r="Z1" s="327" t="n"/>
@@ -9247,12 +9210,12 @@
       <c r="AH1" s="327" t="n"/>
       <c r="AI1" s="327" t="n"/>
       <c r="AJ1" s="327" t="n"/>
-      <c r="AK1" s="327" t="n"/>
-      <c r="AL1" s="328" t="inlineStr">
+      <c r="AK1" s="328" t="inlineStr">
         <is>
           <t>工具特定属性</t>
         </is>
       </c>
+      <c r="AL1" s="329" t="n"/>
       <c r="AM1" s="329" t="n"/>
       <c r="AN1" s="329" t="n"/>
       <c r="AO1" s="329" t="n"/>
@@ -9270,28 +9233,27 @@
       <c r="BA1" s="329" t="n"/>
       <c r="BB1" s="329" t="n"/>
       <c r="BC1" s="329" t="n"/>
-      <c r="BD1" s="329" t="n"/>
-      <c r="BE1" s="330" t="inlineStr">
+      <c r="BD1" s="330" t="inlineStr">
         <is>
           <t>温室气体排放基础</t>
         </is>
       </c>
-      <c r="BF1" s="331" t="n"/>
-      <c r="BG1" s="332" t="inlineStr">
+      <c r="BE1" s="331" t="n"/>
+      <c r="BF1" s="332" t="inlineStr">
         <is>
           <t>分类与指标</t>
         </is>
       </c>
+      <c r="BG1" s="329" t="n"/>
       <c r="BH1" s="329" t="n"/>
       <c r="BI1" s="329" t="n"/>
-      <c r="BJ1" s="329" t="n"/>
-      <c r="BK1" s="333" t="inlineStr">
+      <c r="BJ1" s="333" t="inlineStr">
         <is>
           <t>立法参考</t>
         </is>
       </c>
+      <c r="BK1" s="327" t="n"/>
       <c r="BL1" s="327" t="n"/>
-      <c r="BM1" s="327" t="n"/>
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="334" t="inlineStr">
@@ -9356,282 +9318,277 @@
       </c>
       <c r="M2" s="337" t="inlineStr">
         <is>
-          <t>国家</t>
+          <t>管辖层级</t>
         </is>
       </c>
       <c r="N2" s="337" t="inlineStr">
         <is>
-          <t>管辖层级</t>
+          <t>管辖地名称</t>
         </is>
       </c>
       <c r="O2" s="337" t="inlineStr">
         <is>
-          <t>管辖地名称</t>
+          <t>通过日期</t>
         </is>
       </c>
       <c r="P2" s="337" t="inlineStr">
         <is>
-          <t>通过日期</t>
+          <t>生效日期</t>
         </is>
       </c>
       <c r="Q2" s="337" t="inlineStr">
         <is>
-          <t>生效日期</t>
+          <t>终止日期</t>
         </is>
       </c>
       <c r="R2" s="337" t="inlineStr">
         <is>
-          <t>终止日期</t>
+          <t>最近修订</t>
         </is>
       </c>
       <c r="S2" s="337" t="inlineStr">
         <is>
-          <t>最近修订</t>
+          <t>最近修订（详情）</t>
         </is>
       </c>
       <c r="T2" s="337" t="inlineStr">
         <is>
-          <t>最近修订（详情）</t>
+          <t>状态</t>
         </is>
       </c>
       <c r="U2" s="337" t="inlineStr">
         <is>
-          <t>状态</t>
-        </is>
-      </c>
-      <c r="V2" s="337" t="inlineStr">
-        <is>
           <t>管理机构</t>
         </is>
       </c>
+      <c r="V2" s="338" t="inlineStr">
+        <is>
+          <t>受规制资产</t>
+        </is>
+      </c>
       <c r="W2" s="338" t="inlineStr">
         <is>
-          <t>受规制资产</t>
+          <t>受规制资产（状态）</t>
         </is>
       </c>
       <c r="X2" s="338" t="inlineStr">
         <is>
-          <t>受规制资产（状态）</t>
+          <t>受规制资产（详情）</t>
         </is>
       </c>
       <c r="Y2" s="338" t="inlineStr">
         <is>
-          <t>受规制资产（详情）</t>
+          <t>受规制资产（其他）</t>
         </is>
       </c>
       <c r="Z2" s="338" t="inlineStr">
         <is>
-          <t>受规制资产（其他）</t>
+          <t>受规制资产（阈值范围）</t>
         </is>
       </c>
       <c r="AA2" s="338" t="inlineStr">
         <is>
-          <t>受规制资产（阈值范围）</t>
+          <t>受规制主体</t>
         </is>
       </c>
       <c r="AB2" s="338" t="inlineStr">
         <is>
-          <t>受规制主体</t>
+          <t>受规制主体（详情）</t>
         </is>
       </c>
       <c r="AC2" s="338" t="inlineStr">
         <is>
-          <t>受规制主体（详情）</t>
+          <t>受规制活动</t>
         </is>
       </c>
       <c r="AD2" s="338" t="inlineStr">
         <is>
-          <t>受规制活动</t>
+          <t>受规制活动（详情）</t>
         </is>
       </c>
       <c r="AE2" s="338" t="inlineStr">
         <is>
-          <t>受规制活动（详情）</t>
+          <t>强度（数值）</t>
         </is>
       </c>
       <c r="AF2" s="338" t="inlineStr">
         <is>
-          <t>强度（数值）</t>
+          <t>强度（单位）</t>
         </is>
       </c>
       <c r="AG2" s="338" t="inlineStr">
         <is>
-          <t>强度（单位）</t>
+          <t>强度（详情）</t>
         </is>
       </c>
       <c r="AH2" s="338" t="inlineStr">
         <is>
-          <t>强度（详情）</t>
+          <t>要求说明</t>
         </is>
       </c>
       <c r="AI2" s="338" t="inlineStr">
         <is>
-          <t>要求说明</t>
+          <t>合规计算方法I</t>
         </is>
       </c>
       <c r="AJ2" s="338" t="inlineStr">
         <is>
-          <t>合规计算方法I</t>
-        </is>
-      </c>
-      <c r="AK2" s="338" t="inlineStr">
-        <is>
           <t>合规计算方法II</t>
         </is>
       </c>
+      <c r="AK2" s="339" t="inlineStr">
+        <is>
+          <t>税收及激励：年度收入</t>
+        </is>
+      </c>
       <c r="AL2" s="339" t="inlineStr">
         <is>
-          <t>税收及激励：年度收入</t>
+          <t>税收及激励：专项资金</t>
         </is>
       </c>
       <c r="AM2" s="339" t="inlineStr">
         <is>
-          <t>税收及激励：专项资金</t>
+          <t>税收及激励：年度收入减免</t>
         </is>
       </c>
       <c r="AN2" s="339" t="inlineStr">
         <is>
-          <t>税收及激励：年度收入减免</t>
+          <t>补贴：年度预算/支出</t>
         </is>
       </c>
       <c r="AO2" s="339" t="inlineStr">
         <is>
-          <t>补贴：年度预算/支出</t>
+          <t>补贴：限额</t>
         </is>
       </c>
       <c r="AP2" s="339" t="inlineStr">
         <is>
-          <t>补贴：限额</t>
+          <t>补贴：下限或上限</t>
         </is>
       </c>
       <c r="AQ2" s="339" t="inlineStr">
         <is>
-          <t>补贴：下限或上限</t>
+          <t>补贴：分配机制</t>
         </is>
       </c>
       <c r="AR2" s="339" t="inlineStr">
         <is>
-          <t>补贴：分配机制</t>
+          <t>补贴：支持期限</t>
         </is>
       </c>
       <c r="AS2" s="339" t="inlineStr">
         <is>
-          <t>补贴：支持期限</t>
+          <t>补贴：执行机制</t>
         </is>
       </c>
       <c r="AT2" s="339" t="inlineStr">
         <is>
-          <t>补贴：执行机制</t>
+          <t>交易系统：类型</t>
         </is>
       </c>
       <c r="AU2" s="339" t="inlineStr">
         <is>
-          <t>交易系统：类型</t>
+          <t>交易系统：总量上限</t>
         </is>
       </c>
       <c r="AV2" s="339" t="inlineStr">
         <is>
-          <t>交易系统：总量上限</t>
+          <t>交易系统：配额分配机制</t>
         </is>
       </c>
       <c r="AW2" s="339" t="inlineStr">
         <is>
-          <t>交易系统：配额分配机制</t>
+          <t>交易系统：免费配额</t>
         </is>
       </c>
       <c r="AX2" s="339" t="inlineStr">
         <is>
-          <t>交易系统：免费配额</t>
+          <t>交易系统：允许使用抵消</t>
         </is>
       </c>
       <c r="AY2" s="339" t="inlineStr">
         <is>
-          <t>交易系统：允许使用抵消</t>
+          <t>交易系统：链接</t>
         </is>
       </c>
       <c r="AZ2" s="339" t="inlineStr">
         <is>
-          <t>交易系统：链接</t>
+          <t>交易系统：市场稳定机制</t>
         </is>
       </c>
       <c r="BA2" s="339" t="inlineStr">
         <is>
-          <t>交易系统：市场稳定机制</t>
+          <t>交易系统：年收入</t>
         </is>
       </c>
       <c r="BB2" s="339" t="inlineStr">
         <is>
-          <t>交易系统：年收入</t>
+          <t>交易系统：交易量</t>
         </is>
       </c>
       <c r="BC2" s="339" t="inlineStr">
         <is>
-          <t>交易系统：交易量</t>
-        </is>
-      </c>
-      <c r="BD2" s="339" t="inlineStr">
-        <is>
           <t>交易系统：违规处罚</t>
         </is>
       </c>
+      <c r="BD2" s="340" t="inlineStr">
+        <is>
+          <t>温室气体排放覆盖（绝对量）</t>
+        </is>
+      </c>
       <c r="BE2" s="340" t="inlineStr">
         <is>
-          <t>温室气体排放覆盖（绝对量）</t>
-        </is>
-      </c>
-      <c r="BF2" s="340" t="inlineStr">
-        <is>
           <t>温室气体排放覆盖（占国内排放百分比）</t>
         </is>
       </c>
+      <c r="BF2" s="335" t="inlineStr">
+        <is>
+          <t>经济行业</t>
+        </is>
+      </c>
       <c r="BG2" s="335" t="inlineStr">
         <is>
-          <t>经济行业</t>
+          <t>受影响的温室气体</t>
         </is>
       </c>
       <c r="BH2" s="335" t="inlineStr">
         <is>
-          <t>受影响的温室气体</t>
+          <t>减缓效果</t>
         </is>
       </c>
       <c r="BI2" s="335" t="inlineStr">
         <is>
-          <t>减缓效果</t>
-        </is>
-      </c>
-      <c r="BJ2" s="335" t="inlineStr">
-        <is>
           <t>减缓协同效益</t>
         </is>
       </c>
+      <c r="BJ2" s="337" t="inlineStr">
+        <is>
+          <t>法律文件名称</t>
+        </is>
+      </c>
       <c r="BK2" s="337" t="inlineStr">
         <is>
-          <t>法律文件名称</t>
+          <t>法律文件链接</t>
         </is>
       </c>
       <c r="BL2" s="337" t="inlineStr">
         <is>
-          <t>法律文件链接</t>
-        </is>
-      </c>
-      <c r="BM2" s="337" t="inlineStr">
-        <is>
           <t>其他网页链接</t>
         </is>
       </c>
-      <c r="BN2" s="341" t="n"/>
+      <c r="BM2" s="341" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="G1:L1"/>
-    <mergeCell ref="BK1:BM1"/>
-    <mergeCell ref="AL1:BD1"/>
-    <mergeCell ref="M1:V1"/>
-    <mergeCell ref="BE1:BF1"/>
-    <mergeCell ref="W1:AK1"/>
+    <mergeCell ref="AK1:BC1"/>
+    <mergeCell ref="BJ1:BL1"/>
+    <mergeCell ref="V1:AJ1"/>
+    <mergeCell ref="BF1:BI1"/>
+    <mergeCell ref="BD1:BE1"/>
+    <mergeCell ref="M1:U1"/>
     <mergeCell ref="C1:F1"/>
     <mergeCell ref="A1:B1"/>
-    <mergeCell ref="BG1:BJ1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>
@@ -9736,7 +9693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA2"/>
+  <dimension ref="A1:AZ2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
@@ -9768,12 +9725,12 @@
       <c r="S1" s="344" t="n"/>
       <c r="T1" s="344" t="n"/>
       <c r="U1" s="344" t="n"/>
-      <c r="V1" s="344" t="n"/>
-      <c r="W1" s="345" t="inlineStr">
+      <c r="V1" s="345" t="inlineStr">
         <is>
           <t>政策规制基础与强度</t>
         </is>
       </c>
+      <c r="W1" s="344" t="n"/>
       <c r="X1" s="344" t="n"/>
       <c r="Y1" s="344" t="n"/>
       <c r="Z1" s="344" t="n"/>
@@ -9787,38 +9744,37 @@
       <c r="AH1" s="344" t="n"/>
       <c r="AI1" s="344" t="n"/>
       <c r="AJ1" s="344" t="n"/>
-      <c r="AK1" s="344" t="n"/>
-      <c r="AL1" s="346" t="inlineStr">
+      <c r="AK1" s="346" t="inlineStr">
         <is>
           <t>工具特定属性</t>
         </is>
       </c>
+      <c r="AL1" s="344" t="n"/>
       <c r="AM1" s="344" t="n"/>
       <c r="AN1" s="344" t="n"/>
       <c r="AO1" s="344" t="n"/>
       <c r="AP1" s="344" t="n"/>
-      <c r="AQ1" s="344" t="n"/>
-      <c r="AR1" s="347" t="inlineStr">
+      <c r="AQ1" s="347" t="inlineStr">
         <is>
           <t>温室气体排放基础</t>
         </is>
       </c>
-      <c r="AS1" s="348" t="n"/>
-      <c r="AT1" s="349" t="inlineStr">
+      <c r="AR1" s="348" t="n"/>
+      <c r="AS1" s="349" t="inlineStr">
         <is>
           <t>分类与指标</t>
         </is>
       </c>
+      <c r="AT1" s="344" t="n"/>
       <c r="AU1" s="344" t="n"/>
       <c r="AV1" s="344" t="n"/>
-      <c r="AW1" s="344" t="n"/>
-      <c r="AX1" s="350" t="inlineStr">
+      <c r="AW1" s="350" t="inlineStr">
         <is>
           <t>立法参考</t>
         </is>
       </c>
+      <c r="AX1" s="344" t="n"/>
       <c r="AY1" s="344" t="n"/>
-      <c r="AZ1" s="344" t="n"/>
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="334" t="inlineStr">
@@ -9883,217 +9839,212 @@
       </c>
       <c r="M2" s="351" t="inlineStr">
         <is>
-          <t>国家</t>
+          <t>管辖层级</t>
         </is>
       </c>
       <c r="N2" s="351" t="inlineStr">
         <is>
-          <t>管辖层级</t>
+          <t>管辖地名称</t>
         </is>
       </c>
       <c r="O2" s="351" t="inlineStr">
         <is>
-          <t>管辖地名称</t>
+          <t>通过日期</t>
         </is>
       </c>
       <c r="P2" s="351" t="inlineStr">
         <is>
-          <t>通过日期</t>
+          <t>生效日期</t>
         </is>
       </c>
       <c r="Q2" s="351" t="inlineStr">
         <is>
-          <t>生效日期</t>
+          <t>终止日期</t>
         </is>
       </c>
       <c r="R2" s="351" t="inlineStr">
         <is>
-          <t>终止日期</t>
+          <t>最近修订</t>
         </is>
       </c>
       <c r="S2" s="351" t="inlineStr">
         <is>
-          <t>最近修订</t>
+          <t>最近修订（详情）</t>
         </is>
       </c>
       <c r="T2" s="351" t="inlineStr">
         <is>
-          <t>最近修订（详情）</t>
+          <t>状态</t>
         </is>
       </c>
       <c r="U2" s="351" t="inlineStr">
         <is>
-          <t>状态</t>
-        </is>
-      </c>
-      <c r="V2" s="351" t="inlineStr">
-        <is>
           <t>管理机构</t>
         </is>
       </c>
+      <c r="V2" s="338" t="inlineStr">
+        <is>
+          <t>受规制资产</t>
+        </is>
+      </c>
       <c r="W2" s="338" t="inlineStr">
         <is>
-          <t>受规制资产</t>
+          <t>受规制资产（状态）</t>
         </is>
       </c>
       <c r="X2" s="338" t="inlineStr">
         <is>
-          <t>受规制资产（状态）</t>
+          <t>受规制资产（详情）</t>
         </is>
       </c>
       <c r="Y2" s="338" t="inlineStr">
         <is>
-          <t>受规制资产（详情）</t>
+          <t>受规制资产（其他）</t>
         </is>
       </c>
       <c r="Z2" s="338" t="inlineStr">
         <is>
-          <t>受规制资产（其他）</t>
+          <t>受规制资产（阈值范围）</t>
         </is>
       </c>
       <c r="AA2" s="338" t="inlineStr">
         <is>
-          <t>受规制资产（阈值范围）</t>
+          <t>受规制主体</t>
         </is>
       </c>
       <c r="AB2" s="338" t="inlineStr">
         <is>
-          <t>受规制主体</t>
+          <t>受规制主体（详情）</t>
         </is>
       </c>
       <c r="AC2" s="338" t="inlineStr">
         <is>
-          <t>受规制主体（详情）</t>
+          <t>受规制活动</t>
         </is>
       </c>
       <c r="AD2" s="338" t="inlineStr">
         <is>
-          <t>受规制活动</t>
+          <t>受规制活动（详情）</t>
         </is>
       </c>
       <c r="AE2" s="338" t="inlineStr">
         <is>
-          <t>受规制活动（详情）</t>
+          <t>强度（数值）</t>
         </is>
       </c>
       <c r="AF2" s="338" t="inlineStr">
         <is>
-          <t>强度（数值）</t>
+          <t>强度（单位）</t>
         </is>
       </c>
       <c r="AG2" s="338" t="inlineStr">
         <is>
-          <t>强度（单位）</t>
+          <t>强度（详情）</t>
         </is>
       </c>
       <c r="AH2" s="338" t="inlineStr">
         <is>
-          <t>强度（详情）</t>
+          <t>要求说明</t>
         </is>
       </c>
       <c r="AI2" s="338" t="inlineStr">
         <is>
-          <t>要求说明</t>
+          <t>合规计算方法I</t>
         </is>
       </c>
       <c r="AJ2" s="338" t="inlineStr">
         <is>
-          <t>合规计算方法I</t>
-        </is>
-      </c>
-      <c r="AK2" s="338" t="inlineStr">
-        <is>
           <t>合规计算方法II</t>
         </is>
       </c>
+      <c r="AK2" s="336" t="inlineStr">
+        <is>
+          <t>合规监测</t>
+        </is>
+      </c>
       <c r="AL2" s="336" t="inlineStr">
         <is>
-          <t>合规监测</t>
+          <t>合规监测详情</t>
         </is>
       </c>
       <c r="AM2" s="336" t="inlineStr">
         <is>
-          <t>合规监测详情</t>
+          <t>合规执行</t>
         </is>
       </c>
       <c r="AN2" s="336" t="inlineStr">
         <is>
-          <t>合规执行</t>
+          <t>合规执行详情</t>
         </is>
       </c>
       <c r="AO2" s="336" t="inlineStr">
         <is>
-          <t>合规执行详情</t>
+          <t>合规促进</t>
         </is>
       </c>
       <c r="AP2" s="336" t="inlineStr">
         <is>
-          <t>合规促进</t>
-        </is>
-      </c>
-      <c r="AQ2" s="336" t="inlineStr">
-        <is>
           <t>合规促进详情</t>
         </is>
       </c>
+      <c r="AQ2" s="340" t="inlineStr">
+        <is>
+          <t>温室气体排放覆盖（绝对量）</t>
+        </is>
+      </c>
       <c r="AR2" s="340" t="inlineStr">
         <is>
-          <t>温室气体排放覆盖（绝对量）</t>
-        </is>
-      </c>
-      <c r="AS2" s="340" t="inlineStr">
-        <is>
           <t>温室气体排放覆盖（占国内排放百分比）</t>
         </is>
       </c>
+      <c r="AS2" s="352" t="inlineStr">
+        <is>
+          <t>经济行业</t>
+        </is>
+      </c>
       <c r="AT2" s="352" t="inlineStr">
         <is>
-          <t>经济行业</t>
+          <t>受影响的温室气体</t>
         </is>
       </c>
       <c r="AU2" s="352" t="inlineStr">
         <is>
-          <t>受影响的温室气体</t>
+          <t>减缓效果</t>
         </is>
       </c>
       <c r="AV2" s="352" t="inlineStr">
         <is>
-          <t>减缓效果</t>
-        </is>
-      </c>
-      <c r="AW2" s="352" t="inlineStr">
-        <is>
           <t>减缓协同效益</t>
         </is>
       </c>
+      <c r="AW2" s="337" t="inlineStr">
+        <is>
+          <t>法律文件名称</t>
+        </is>
+      </c>
       <c r="AX2" s="337" t="inlineStr">
         <is>
-          <t>法律文件名称</t>
+          <t>法律文件链接</t>
         </is>
       </c>
       <c r="AY2" s="337" t="inlineStr">
         <is>
-          <t>法律文件链接</t>
-        </is>
-      </c>
-      <c r="AZ2" s="337" t="inlineStr">
-        <is>
           <t>其他网页链接</t>
         </is>
       </c>
-      <c r="BA2" s="341" t="n"/>
+      <c r="AZ2" s="341" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="G1:L1"/>
-    <mergeCell ref="AX1:AZ1"/>
-    <mergeCell ref="M1:V1"/>
-    <mergeCell ref="AL1:AQ1"/>
-    <mergeCell ref="AR1:AS1"/>
-    <mergeCell ref="W1:AK1"/>
+    <mergeCell ref="V1:AJ1"/>
+    <mergeCell ref="AK1:AP1"/>
+    <mergeCell ref="AW1:AY1"/>
+    <mergeCell ref="M1:U1"/>
     <mergeCell ref="C1:F1"/>
+    <mergeCell ref="AQ1:AR1"/>
     <mergeCell ref="A1:B1"/>
-    <mergeCell ref="AT1:AW1"/>
+    <mergeCell ref="AS1:AV1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -10105,7 +10056,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BC2"/>
+  <dimension ref="A1:BB2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
@@ -10137,12 +10088,12 @@
       <c r="S1" s="329" t="n"/>
       <c r="T1" s="329" t="n"/>
       <c r="U1" s="329" t="n"/>
-      <c r="V1" s="329" t="n"/>
-      <c r="W1" s="354" t="inlineStr">
+      <c r="V1" s="354" t="inlineStr">
         <is>
           <t>政策规制基础与强度</t>
         </is>
       </c>
+      <c r="W1" s="329" t="n"/>
       <c r="X1" s="329" t="n"/>
       <c r="Y1" s="329" t="n"/>
       <c r="Z1" s="329" t="n"/>
@@ -10156,40 +10107,39 @@
       <c r="AH1" s="329" t="n"/>
       <c r="AI1" s="329" t="n"/>
       <c r="AJ1" s="329" t="n"/>
-      <c r="AK1" s="329" t="n"/>
-      <c r="AL1" s="328" t="inlineStr">
+      <c r="AK1" s="328" t="inlineStr">
         <is>
           <t>工具特定属性</t>
         </is>
       </c>
+      <c r="AL1" s="329" t="n"/>
       <c r="AM1" s="329" t="n"/>
       <c r="AN1" s="329" t="n"/>
       <c r="AO1" s="329" t="n"/>
       <c r="AP1" s="329" t="n"/>
       <c r="AQ1" s="329" t="n"/>
       <c r="AR1" s="329" t="n"/>
-      <c r="AS1" s="329" t="n"/>
-      <c r="AT1" s="355" t="inlineStr">
+      <c r="AS1" s="355" t="inlineStr">
         <is>
           <t>温室气体排放基础</t>
         </is>
       </c>
-      <c r="AU1" s="331" t="n"/>
-      <c r="AV1" s="332" t="inlineStr">
+      <c r="AT1" s="331" t="n"/>
+      <c r="AU1" s="332" t="inlineStr">
         <is>
           <t>分类与指标</t>
         </is>
       </c>
+      <c r="AV1" s="329" t="n"/>
       <c r="AW1" s="329" t="n"/>
       <c r="AX1" s="329" t="n"/>
-      <c r="AY1" s="329" t="n"/>
-      <c r="AZ1" s="353" t="inlineStr">
+      <c r="AY1" s="353" t="inlineStr">
         <is>
           <t>立法参考</t>
         </is>
       </c>
+      <c r="AZ1" s="329" t="n"/>
       <c r="BA1" s="329" t="n"/>
-      <c r="BB1" s="329" t="n"/>
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="334" t="inlineStr">
@@ -10254,227 +10204,222 @@
       </c>
       <c r="M2" s="337" t="inlineStr">
         <is>
-          <t>国家</t>
+          <t>管辖层级</t>
         </is>
       </c>
       <c r="N2" s="337" t="inlineStr">
         <is>
-          <t>管辖层级</t>
+          <t>管辖地名称</t>
         </is>
       </c>
       <c r="O2" s="337" t="inlineStr">
         <is>
-          <t>管辖地名称</t>
+          <t>通过日期</t>
         </is>
       </c>
       <c r="P2" s="337" t="inlineStr">
         <is>
-          <t>通过日期</t>
+          <t>生效日期</t>
         </is>
       </c>
       <c r="Q2" s="337" t="inlineStr">
         <is>
-          <t>生效日期</t>
+          <t>终止日期</t>
         </is>
       </c>
       <c r="R2" s="337" t="inlineStr">
         <is>
-          <t>终止日期</t>
+          <t>最近修订</t>
         </is>
       </c>
       <c r="S2" s="337" t="inlineStr">
         <is>
-          <t>最近修订</t>
+          <t>最近修订（详情）</t>
         </is>
       </c>
       <c r="T2" s="337" t="inlineStr">
         <is>
-          <t>最近修订（详情）</t>
+          <t>状态</t>
         </is>
       </c>
       <c r="U2" s="337" t="inlineStr">
         <is>
-          <t>状态</t>
-        </is>
-      </c>
-      <c r="V2" s="337" t="inlineStr">
-        <is>
           <t>管理机构</t>
         </is>
       </c>
+      <c r="V2" s="338" t="inlineStr">
+        <is>
+          <t>受规制资产</t>
+        </is>
+      </c>
       <c r="W2" s="338" t="inlineStr">
         <is>
-          <t>受规制资产</t>
+          <t>受规制资产（状态）</t>
         </is>
       </c>
       <c r="X2" s="338" t="inlineStr">
         <is>
-          <t>受规制资产（状态）</t>
+          <t>受规制资产（详情）</t>
         </is>
       </c>
       <c r="Y2" s="338" t="inlineStr">
         <is>
-          <t>受规制资产（详情）</t>
+          <t>受规制资产（其他）</t>
         </is>
       </c>
       <c r="Z2" s="338" t="inlineStr">
         <is>
-          <t>受规制资产（其他）</t>
+          <t>受规制资产（阈值范围）</t>
         </is>
       </c>
       <c r="AA2" s="338" t="inlineStr">
         <is>
-          <t>受规制资产（阈值范围）</t>
+          <t>受规制主体</t>
         </is>
       </c>
       <c r="AB2" s="338" t="inlineStr">
         <is>
-          <t>受规制主体</t>
+          <t>受规制主体（详情）</t>
         </is>
       </c>
       <c r="AC2" s="338" t="inlineStr">
         <is>
-          <t>受规制主体（详情）</t>
+          <t>受规制活动</t>
         </is>
       </c>
       <c r="AD2" s="338" t="inlineStr">
         <is>
-          <t>受规制活动</t>
+          <t>受规制活动（详情）</t>
         </is>
       </c>
       <c r="AE2" s="338" t="inlineStr">
         <is>
-          <t>受规制活动（详情）</t>
+          <t>强度（数值）</t>
         </is>
       </c>
       <c r="AF2" s="338" t="inlineStr">
         <is>
-          <t>强度（数值）</t>
+          <t>强度（单位）</t>
         </is>
       </c>
       <c r="AG2" s="338" t="inlineStr">
         <is>
-          <t>强度（单位）</t>
+          <t>强度（详情）</t>
         </is>
       </c>
       <c r="AH2" s="338" t="inlineStr">
         <is>
-          <t>强度（详情）</t>
+          <t>要求说明</t>
         </is>
       </c>
       <c r="AI2" s="338" t="inlineStr">
         <is>
-          <t>要求说明</t>
+          <t>合规计算方法I</t>
         </is>
       </c>
       <c r="AJ2" s="338" t="inlineStr">
         <is>
-          <t>合规计算方法I</t>
-        </is>
-      </c>
-      <c r="AK2" s="338" t="inlineStr">
-        <is>
           <t>合规计算方法II</t>
         </is>
       </c>
+      <c r="AK2" s="339" t="inlineStr">
+        <is>
+          <t>公共投资：共同融资</t>
+        </is>
+      </c>
       <c r="AL2" s="339" t="inlineStr">
         <is>
-          <t>公共投资：共同融资</t>
+          <t>公共投资：选择流程</t>
         </is>
       </c>
       <c r="AM2" s="339" t="inlineStr">
         <is>
-          <t>公共投资：选择流程</t>
+          <t>公共采购：招标流程</t>
         </is>
       </c>
       <c r="AN2" s="339" t="inlineStr">
         <is>
-          <t>公共采购：招标流程</t>
+          <t>公共采购：招标评标标准</t>
         </is>
       </c>
       <c r="AO2" s="339" t="inlineStr">
         <is>
-          <t>公共采购：招标评标标准</t>
+          <t>公共采购：合规监测</t>
         </is>
       </c>
       <c r="AP2" s="339" t="inlineStr">
         <is>
-          <t>公共采购：合规监测</t>
+          <t>公共采购：合规执行</t>
         </is>
       </c>
       <c r="AQ2" s="339" t="inlineStr">
         <is>
-          <t>公共采购：合规执行</t>
+          <t>公共采购：全生命周期成本</t>
         </is>
       </c>
       <c r="AR2" s="339" t="inlineStr">
         <is>
-          <t>公共采购：全生命周期成本</t>
-        </is>
-      </c>
-      <c r="AS2" s="339" t="inlineStr">
-        <is>
           <t>公共投资/采购：年度支出</t>
         </is>
       </c>
+      <c r="AS2" s="340" t="inlineStr">
+        <is>
+          <t>温室气体排放覆盖（绝对量）</t>
+        </is>
+      </c>
       <c r="AT2" s="340" t="inlineStr">
         <is>
-          <t>温室气体排放覆盖（绝对量）</t>
-        </is>
-      </c>
-      <c r="AU2" s="340" t="inlineStr">
-        <is>
           <t>温室气体排放覆盖（占国内排放百分比）</t>
         </is>
       </c>
+      <c r="AU2" s="352" t="inlineStr">
+        <is>
+          <t>经济行业</t>
+        </is>
+      </c>
       <c r="AV2" s="352" t="inlineStr">
         <is>
-          <t>经济行业</t>
+          <t>受影响的温室气体</t>
         </is>
       </c>
       <c r="AW2" s="352" t="inlineStr">
         <is>
-          <t>受影响的温室气体</t>
+          <t>减缓效果</t>
         </is>
       </c>
       <c r="AX2" s="352" t="inlineStr">
         <is>
-          <t>减缓效果</t>
-        </is>
-      </c>
-      <c r="AY2" s="352" t="inlineStr">
-        <is>
           <t>减缓协同效益</t>
         </is>
       </c>
+      <c r="AY2" s="337" t="inlineStr">
+        <is>
+          <t>法律文件名称</t>
+        </is>
+      </c>
       <c r="AZ2" s="337" t="inlineStr">
         <is>
-          <t>法律文件名称</t>
+          <t>法律文件链接</t>
         </is>
       </c>
       <c r="BA2" s="337" t="inlineStr">
         <is>
-          <t>法律文件链接</t>
-        </is>
-      </c>
-      <c r="BB2" s="337" t="inlineStr">
-        <is>
           <t>其他网页链接</t>
         </is>
       </c>
-      <c r="BC2" s="341" t="n"/>
+      <c r="BB2" s="341" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="G1:L1"/>
-    <mergeCell ref="AZ1:BB1"/>
-    <mergeCell ref="M1:V1"/>
-    <mergeCell ref="W1:AK1"/>
-    <mergeCell ref="AV1:AY1"/>
-    <mergeCell ref="AT1:AU1"/>
+    <mergeCell ref="AU1:AX1"/>
+    <mergeCell ref="V1:AJ1"/>
+    <mergeCell ref="AY1:BA1"/>
+    <mergeCell ref="M1:U1"/>
+    <mergeCell ref="AS1:AT1"/>
     <mergeCell ref="C1:F1"/>
     <mergeCell ref="A1:B1"/>
-    <mergeCell ref="AL1:AS1"/>
+    <mergeCell ref="AK1:AR1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -10486,7 +10431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BF2"/>
+  <dimension ref="A1:BE2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
@@ -10518,12 +10463,12 @@
       <c r="S1" s="329" t="n"/>
       <c r="T1" s="329" t="n"/>
       <c r="U1" s="329" t="n"/>
-      <c r="V1" s="329" t="n"/>
-      <c r="W1" s="357" t="inlineStr">
+      <c r="V1" s="357" t="inlineStr">
         <is>
           <t>政策规制基础与强度</t>
         </is>
       </c>
+      <c r="W1" s="329" t="n"/>
       <c r="X1" s="329" t="n"/>
       <c r="Y1" s="329" t="n"/>
       <c r="Z1" s="329" t="n"/>
@@ -10537,12 +10482,12 @@
       <c r="AH1" s="329" t="n"/>
       <c r="AI1" s="329" t="n"/>
       <c r="AJ1" s="329" t="n"/>
-      <c r="AK1" s="329" t="n"/>
-      <c r="AL1" s="358" t="inlineStr">
+      <c r="AK1" s="358" t="inlineStr">
         <is>
           <t>工具特定属性</t>
         </is>
       </c>
+      <c r="AL1" s="327" t="n"/>
       <c r="AM1" s="327" t="n"/>
       <c r="AN1" s="327" t="n"/>
       <c r="AO1" s="327" t="n"/>
@@ -10551,28 +10496,27 @@
       <c r="AR1" s="327" t="n"/>
       <c r="AS1" s="327" t="n"/>
       <c r="AT1" s="327" t="n"/>
-      <c r="AU1" s="327" t="n"/>
-      <c r="AV1" s="359" t="inlineStr">
+      <c r="AU1" s="359" t="inlineStr">
         <is>
           <t>温室气体排放基础</t>
         </is>
       </c>
-      <c r="AW1" s="327" t="n"/>
-      <c r="AX1" s="357" t="inlineStr">
+      <c r="AV1" s="327" t="n"/>
+      <c r="AW1" s="357" t="inlineStr">
         <is>
           <t>分类与指标</t>
         </is>
       </c>
+      <c r="AX1" s="329" t="n"/>
       <c r="AY1" s="329" t="n"/>
       <c r="AZ1" s="329" t="n"/>
-      <c r="BA1" s="329" t="n"/>
-      <c r="BB1" s="360" t="inlineStr">
+      <c r="BA1" s="360" t="inlineStr">
         <is>
           <t>立法参考</t>
         </is>
       </c>
-      <c r="BC1" s="329" t="n"/>
-      <c r="BD1" s="361" t="n"/>
+      <c r="BB1" s="329" t="n"/>
+      <c r="BC1" s="361" t="n"/>
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="334" t="inlineStr">
@@ -10637,238 +10581,233 @@
       </c>
       <c r="M2" s="337" t="inlineStr">
         <is>
-          <t>国家</t>
+          <t>管辖层级</t>
         </is>
       </c>
       <c r="N2" s="337" t="inlineStr">
         <is>
-          <t>管辖层级</t>
+          <t>管辖地名称</t>
         </is>
       </c>
       <c r="O2" s="337" t="inlineStr">
         <is>
-          <t>管辖地名称</t>
+          <t>通过日期</t>
         </is>
       </c>
       <c r="P2" s="337" t="inlineStr">
         <is>
-          <t>通过日期</t>
+          <t>生效日期</t>
         </is>
       </c>
       <c r="Q2" s="337" t="inlineStr">
         <is>
-          <t>生效日期</t>
+          <t>终止日期</t>
         </is>
       </c>
       <c r="R2" s="337" t="inlineStr">
         <is>
-          <t>终止日期</t>
+          <t>最近修订</t>
         </is>
       </c>
       <c r="S2" s="337" t="inlineStr">
         <is>
-          <t>最近修订</t>
+          <t>最近修订（详情）</t>
         </is>
       </c>
       <c r="T2" s="337" t="inlineStr">
         <is>
-          <t>最近修订（详情）</t>
+          <t>状态</t>
         </is>
       </c>
       <c r="U2" s="337" t="inlineStr">
         <is>
-          <t>状态</t>
-        </is>
-      </c>
-      <c r="V2" s="337" t="inlineStr">
-        <is>
           <t>管理机构</t>
         </is>
       </c>
+      <c r="V2" s="338" t="inlineStr">
+        <is>
+          <t>受规制资产</t>
+        </is>
+      </c>
       <c r="W2" s="338" t="inlineStr">
         <is>
-          <t>受规制资产</t>
+          <t>受规制资产（状态）</t>
         </is>
       </c>
       <c r="X2" s="338" t="inlineStr">
         <is>
-          <t>受规制资产（状态）</t>
+          <t>受规制资产（详情）</t>
         </is>
       </c>
       <c r="Y2" s="338" t="inlineStr">
         <is>
-          <t>受规制资产（详情）</t>
+          <t>受规制资产（其他）</t>
         </is>
       </c>
       <c r="Z2" s="338" t="inlineStr">
         <is>
-          <t>受规制资产（其他）</t>
+          <t>受规制资产（阈值范围）</t>
         </is>
       </c>
       <c r="AA2" s="338" t="inlineStr">
         <is>
-          <t>受规制资产（阈值范围）</t>
+          <t>受规制主体</t>
         </is>
       </c>
       <c r="AB2" s="338" t="inlineStr">
         <is>
-          <t>受规制主体</t>
+          <t>受规制主体（详情）</t>
         </is>
       </c>
       <c r="AC2" s="338" t="inlineStr">
         <is>
-          <t>受规制主体（详情）</t>
+          <t>受规制活动</t>
         </is>
       </c>
       <c r="AD2" s="338" t="inlineStr">
         <is>
-          <t>受规制活动</t>
+          <t>受规制活动（详情）</t>
         </is>
       </c>
       <c r="AE2" s="338" t="inlineStr">
         <is>
-          <t>受规制活动（详情）</t>
+          <t>强度（数值）</t>
         </is>
       </c>
       <c r="AF2" s="338" t="inlineStr">
         <is>
-          <t>强度（数值）</t>
+          <t>强度（单位）</t>
         </is>
       </c>
       <c r="AG2" s="338" t="inlineStr">
         <is>
-          <t>强度（单位）</t>
+          <t>强度（详情）</t>
         </is>
       </c>
       <c r="AH2" s="338" t="inlineStr">
         <is>
-          <t>强度（详情）</t>
+          <t>要求说明</t>
         </is>
       </c>
       <c r="AI2" s="338" t="inlineStr">
         <is>
-          <t>要求说明</t>
+          <t>合规计算方法I</t>
         </is>
       </c>
       <c r="AJ2" s="338" t="inlineStr">
         <is>
-          <t>合规计算方法I</t>
-        </is>
-      </c>
-      <c r="AK2" s="338" t="inlineStr">
-        <is>
           <t>合规计算方法II</t>
         </is>
       </c>
+      <c r="AK2" s="339" t="inlineStr">
+        <is>
+          <t>工具联动</t>
+        </is>
+      </c>
       <c r="AL2" s="339" t="inlineStr">
         <is>
-          <t>工具联动</t>
+          <t>信息采集责任方</t>
         </is>
       </c>
       <c r="AM2" s="339" t="inlineStr">
         <is>
-          <t>信息采集责任方</t>
+          <t>信息传输方式</t>
         </is>
       </c>
       <c r="AN2" s="339" t="inlineStr">
         <is>
-          <t>信息传输方式</t>
+          <t>信息提供频率</t>
         </is>
       </c>
       <c r="AO2" s="339" t="inlineStr">
         <is>
-          <t>信息提供频率</t>
+          <t>信息公开可用性</t>
         </is>
       </c>
       <c r="AP2" s="339" t="inlineStr">
         <is>
-          <t>信息公开可用性</t>
+          <t>标签类型</t>
         </is>
       </c>
       <c r="AQ2" s="339" t="inlineStr">
         <is>
-          <t>标签类型</t>
+          <t>合规监测</t>
         </is>
       </c>
       <c r="AR2" s="339" t="inlineStr">
         <is>
-          <t>合规监测</t>
+          <t>合规执行</t>
         </is>
       </c>
       <c r="AS2" s="339" t="inlineStr">
         <is>
-          <t>合规执行</t>
+          <t>合规促进</t>
         </is>
       </c>
       <c r="AT2" s="339" t="inlineStr">
         <is>
-          <t>合规促进</t>
-        </is>
-      </c>
-      <c r="AU2" s="339" t="inlineStr">
-        <is>
           <t>能力建设、培训/教育、宣传和奖励计划详情</t>
         </is>
       </c>
+      <c r="AU2" s="362" t="inlineStr">
+        <is>
+          <t>温室气体排放覆盖（绝对量）</t>
+        </is>
+      </c>
       <c r="AV2" s="362" t="inlineStr">
         <is>
-          <t>温室气体排放覆盖（绝对量）</t>
-        </is>
-      </c>
-      <c r="AW2" s="362" t="inlineStr">
-        <is>
           <t>温室气体排放覆盖（占国内排放百分比）</t>
         </is>
       </c>
+      <c r="AW2" s="335" t="inlineStr">
+        <is>
+          <t>经济行业</t>
+        </is>
+      </c>
       <c r="AX2" s="335" t="inlineStr">
         <is>
-          <t>经济行业</t>
+          <t>受影响的温室气体</t>
         </is>
       </c>
       <c r="AY2" s="335" t="inlineStr">
         <is>
-          <t>受影响的温室气体</t>
+          <t>减缓效果</t>
         </is>
       </c>
       <c r="AZ2" s="335" t="inlineStr">
         <is>
-          <t>减缓效果</t>
-        </is>
-      </c>
-      <c r="BA2" s="335" t="inlineStr">
-        <is>
           <t>减缓协同效益</t>
         </is>
       </c>
+      <c r="BA2" s="337" t="inlineStr">
+        <is>
+          <t>法律文件名称</t>
+        </is>
+      </c>
       <c r="BB2" s="337" t="inlineStr">
         <is>
-          <t>法律文件名称</t>
+          <t>法律文件链接</t>
         </is>
       </c>
       <c r="BC2" s="337" t="inlineStr">
         <is>
-          <t>法律文件链接</t>
-        </is>
-      </c>
-      <c r="BD2" s="337" t="inlineStr">
-        <is>
           <t>其他网页链接</t>
         </is>
       </c>
+      <c r="BD2" s="363" t="n"/>
       <c r="BE2" s="363" t="n"/>
-      <c r="BF2" s="363" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="AK1:AT1"/>
     <mergeCell ref="G1:L1"/>
-    <mergeCell ref="AL1:AU1"/>
-    <mergeCell ref="BB1:BD1"/>
-    <mergeCell ref="AV1:AW1"/>
-    <mergeCell ref="M1:V1"/>
-    <mergeCell ref="W1:AK1"/>
+    <mergeCell ref="AW1:AZ1"/>
+    <mergeCell ref="BA1:BC1"/>
+    <mergeCell ref="V1:AJ1"/>
+    <mergeCell ref="M1:U1"/>
     <mergeCell ref="C1:F1"/>
     <mergeCell ref="A1:B1"/>
-    <mergeCell ref="AX1:BA1"/>
+    <mergeCell ref="AU1:AV1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -10880,7 +10819,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX2"/>
+  <dimension ref="A1:AW2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
@@ -10912,12 +10851,12 @@
       <c r="S1" s="329" t="n"/>
       <c r="T1" s="329" t="n"/>
       <c r="U1" s="329" t="n"/>
-      <c r="V1" s="329" t="n"/>
-      <c r="W1" s="354" t="inlineStr">
+      <c r="V1" s="354" t="inlineStr">
         <is>
           <t>政策规制基础与强度</t>
         </is>
       </c>
+      <c r="W1" s="329" t="n"/>
       <c r="X1" s="329" t="n"/>
       <c r="Y1" s="329" t="n"/>
       <c r="Z1" s="329" t="n"/>
@@ -10931,35 +10870,34 @@
       <c r="AH1" s="329" t="n"/>
       <c r="AI1" s="329" t="n"/>
       <c r="AJ1" s="329" t="n"/>
-      <c r="AK1" s="329" t="n"/>
-      <c r="AL1" s="328" t="inlineStr">
+      <c r="AK1" s="328" t="inlineStr">
         <is>
           <t>工具特定属性</t>
         </is>
       </c>
+      <c r="AL1" s="329" t="n"/>
       <c r="AM1" s="329" t="n"/>
-      <c r="AN1" s="329" t="n"/>
-      <c r="AO1" s="355" t="inlineStr">
+      <c r="AN1" s="355" t="inlineStr">
         <is>
           <t>温室气体排放基础</t>
         </is>
       </c>
-      <c r="AP1" s="331" t="n"/>
-      <c r="AQ1" s="332" t="inlineStr">
+      <c r="AO1" s="331" t="n"/>
+      <c r="AP1" s="332" t="inlineStr">
         <is>
           <t>分类与指标</t>
         </is>
       </c>
+      <c r="AQ1" s="329" t="n"/>
       <c r="AR1" s="329" t="n"/>
       <c r="AS1" s="329" t="n"/>
-      <c r="AT1" s="329" t="n"/>
-      <c r="AU1" s="353" t="inlineStr">
+      <c r="AT1" s="353" t="inlineStr">
         <is>
           <t>立法参考</t>
         </is>
       </c>
+      <c r="AU1" s="329" t="n"/>
       <c r="AV1" s="329" t="n"/>
-      <c r="AW1" s="329" t="n"/>
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="334" t="inlineStr">
@@ -11024,202 +10962,197 @@
       </c>
       <c r="M2" s="337" t="inlineStr">
         <is>
-          <t>国家</t>
+          <t>管辖层级</t>
         </is>
       </c>
       <c r="N2" s="337" t="inlineStr">
         <is>
-          <t>管辖层级</t>
+          <t>管辖地名称</t>
         </is>
       </c>
       <c r="O2" s="337" t="inlineStr">
         <is>
-          <t>管辖地名称</t>
+          <t>通过日期</t>
         </is>
       </c>
       <c r="P2" s="337" t="inlineStr">
         <is>
-          <t>通过日期</t>
+          <t>生效日期</t>
         </is>
       </c>
       <c r="Q2" s="337" t="inlineStr">
         <is>
-          <t>生效日期</t>
+          <t>终止日期</t>
         </is>
       </c>
       <c r="R2" s="337" t="inlineStr">
         <is>
-          <t>终止日期</t>
+          <t>最近修订</t>
         </is>
       </c>
       <c r="S2" s="337" t="inlineStr">
         <is>
-          <t>最近修订</t>
+          <t>最近修订（详情）</t>
         </is>
       </c>
       <c r="T2" s="337" t="inlineStr">
         <is>
-          <t>最近修订（详情）</t>
+          <t>状态</t>
         </is>
       </c>
       <c r="U2" s="337" t="inlineStr">
         <is>
-          <t>状态</t>
-        </is>
-      </c>
-      <c r="V2" s="337" t="inlineStr">
-        <is>
           <t>管理机构</t>
         </is>
       </c>
+      <c r="V2" s="338" t="inlineStr">
+        <is>
+          <t>受规制资产</t>
+        </is>
+      </c>
       <c r="W2" s="338" t="inlineStr">
         <is>
-          <t>受规制资产</t>
+          <t>受规制资产（状态）</t>
         </is>
       </c>
       <c r="X2" s="338" t="inlineStr">
         <is>
-          <t>受规制资产（状态）</t>
+          <t>受规制资产（详情）</t>
         </is>
       </c>
       <c r="Y2" s="338" t="inlineStr">
         <is>
-          <t>受规制资产（详情）</t>
+          <t>受规制资产（其他）</t>
         </is>
       </c>
       <c r="Z2" s="338" t="inlineStr">
         <is>
-          <t>受规制资产（其他）</t>
+          <t>受规制资产（阈值范围）</t>
         </is>
       </c>
       <c r="AA2" s="338" t="inlineStr">
         <is>
-          <t>受规制资产（阈值范围）</t>
+          <t>受规制主体</t>
         </is>
       </c>
       <c r="AB2" s="338" t="inlineStr">
         <is>
-          <t>受规制主体</t>
+          <t>受规制主体（详情）</t>
         </is>
       </c>
       <c r="AC2" s="338" t="inlineStr">
         <is>
-          <t>受规制主体（详情）</t>
+          <t>受规制活动</t>
         </is>
       </c>
       <c r="AD2" s="338" t="inlineStr">
         <is>
-          <t>受规制活动</t>
+          <t>受规制活动（详情）</t>
         </is>
       </c>
       <c r="AE2" s="338" t="inlineStr">
         <is>
-          <t>受规制活动（详情）</t>
+          <t>强度（数值）</t>
         </is>
       </c>
       <c r="AF2" s="338" t="inlineStr">
         <is>
-          <t>强度（数值）</t>
+          <t>强度（单位）</t>
         </is>
       </c>
       <c r="AG2" s="338" t="inlineStr">
         <is>
-          <t>强度（单位）</t>
+          <t>强度（详情）</t>
         </is>
       </c>
       <c r="AH2" s="338" t="inlineStr">
         <is>
-          <t>强度（详情）</t>
+          <t>要求说明</t>
         </is>
       </c>
       <c r="AI2" s="338" t="inlineStr">
         <is>
-          <t>要求说明</t>
+          <t>合规计算方法I</t>
         </is>
       </c>
       <c r="AJ2" s="338" t="inlineStr">
         <is>
-          <t>合规计算方法I</t>
-        </is>
-      </c>
-      <c r="AK2" s="338" t="inlineStr">
-        <is>
           <t>合规计算方法II</t>
         </is>
       </c>
+      <c r="AK2" s="336" t="inlineStr">
+        <is>
+          <t>参与激励</t>
+        </is>
+      </c>
       <c r="AL2" s="336" t="inlineStr">
         <is>
-          <t>参与激励</t>
+          <t>监测</t>
         </is>
       </c>
       <c r="AM2" s="336" t="inlineStr">
         <is>
-          <t>监测</t>
-        </is>
-      </c>
-      <c r="AN2" s="336" t="inlineStr">
-        <is>
           <t>违规制裁</t>
         </is>
       </c>
+      <c r="AN2" s="340" t="inlineStr">
+        <is>
+          <t>温室气体排放覆盖（绝对量）</t>
+        </is>
+      </c>
       <c r="AO2" s="340" t="inlineStr">
         <is>
-          <t>温室气体排放覆盖（绝对量）</t>
-        </is>
-      </c>
-      <c r="AP2" s="340" t="inlineStr">
-        <is>
           <t>温室气体排放覆盖（占国内排放百分比）</t>
         </is>
       </c>
+      <c r="AP2" s="335" t="inlineStr">
+        <is>
+          <t>经济行业</t>
+        </is>
+      </c>
       <c r="AQ2" s="335" t="inlineStr">
         <is>
-          <t>经济行业</t>
+          <t>受影响的温室气体</t>
         </is>
       </c>
       <c r="AR2" s="335" t="inlineStr">
         <is>
-          <t>受影响的温室气体</t>
+          <t>减缓效果</t>
         </is>
       </c>
       <c r="AS2" s="335" t="inlineStr">
         <is>
-          <t>减缓效果</t>
-        </is>
-      </c>
-      <c r="AT2" s="335" t="inlineStr">
-        <is>
           <t>减缓协同效益</t>
         </is>
       </c>
+      <c r="AT2" s="337" t="inlineStr">
+        <is>
+          <t>法律文件名称</t>
+        </is>
+      </c>
       <c r="AU2" s="337" t="inlineStr">
         <is>
-          <t>法律文件名称</t>
+          <t>法律文件链接</t>
         </is>
       </c>
       <c r="AV2" s="337" t="inlineStr">
         <is>
-          <t>法律文件链接</t>
-        </is>
-      </c>
-      <c r="AW2" s="337" t="inlineStr">
-        <is>
           <t>其他网页链接</t>
         </is>
       </c>
-      <c r="AX2" s="341" t="n"/>
+      <c r="AW2" s="341" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="AQ1:AT1"/>
     <mergeCell ref="G1:L1"/>
-    <mergeCell ref="AL1:AN1"/>
-    <mergeCell ref="M1:V1"/>
-    <mergeCell ref="AU1:AW1"/>
-    <mergeCell ref="W1:AK1"/>
-    <mergeCell ref="AO1:AP1"/>
+    <mergeCell ref="AK1:AM1"/>
+    <mergeCell ref="V1:AJ1"/>
+    <mergeCell ref="AT1:AV1"/>
+    <mergeCell ref="AN1:AO1"/>
+    <mergeCell ref="M1:U1"/>
     <mergeCell ref="C1:F1"/>
     <mergeCell ref="A1:B1"/>
+    <mergeCell ref="AP1:AS1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>